<commit_message>
Update treasury bond yields - 2026-04-24
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -460,6 +460,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,6 +529,11 @@
           <t>22-Apr-26</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>23-Apr-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -573,6 +579,9 @@
       <c r="M2" s="3" t="n">
         <v>0.08153333333333335</v>
       </c>
+      <c r="N2" s="3" t="n">
+        <v>0.08153333333333335</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -618,6 +627,9 @@
       <c r="M3" s="3" t="n">
         <v>0.08171666666666667</v>
       </c>
+      <c r="N3" s="3" t="n">
+        <v>0.08188333333333335</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -663,6 +675,9 @@
       <c r="M4" s="3" t="n">
         <v>0.08282857142857145</v>
       </c>
+      <c r="N4" s="3" t="n">
+        <v>0.08297142857142858</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -708,6 +723,9 @@
       <c r="M5" s="3" t="n">
         <v>0.08465555555555555</v>
       </c>
+      <c r="N5" s="3" t="n">
+        <v>0.08493333333333335</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -753,6 +771,9 @@
       <c r="M6" s="3" t="n">
         <v>0.08498333333333334</v>
       </c>
+      <c r="N6" s="3" t="n">
+        <v>0.08473333333333333</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -798,6 +819,9 @@
       <c r="M7" s="3" t="n">
         <v>0.08664285714285715</v>
       </c>
+      <c r="N7" s="3" t="n">
+        <v>0.08664285714285715</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -843,6 +867,9 @@
       <c r="M8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="N8" s="3" t="n">
+        <v>0.08629999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -888,6 +915,9 @@
       <c r="M9" s="3" t="n">
         <v>0.08851999999999999</v>
       </c>
+      <c r="N9" s="3" t="n">
+        <v>0.08851999999999999</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -933,6 +963,9 @@
       <c r="M10" s="3" t="n">
         <v>0.08972857142857142</v>
       </c>
+      <c r="N10" s="3" t="n">
+        <v>0.08972857142857142</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -978,6 +1011,9 @@
       <c r="M11" s="3" t="n">
         <v>0.08984</v>
       </c>
+      <c r="N11" s="3" t="n">
+        <v>0.08984</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1023,6 +1059,9 @@
       <c r="M12" s="3" t="n">
         <v>0.09111666666666667</v>
       </c>
+      <c r="N12" s="3" t="n">
+        <v>0.09111666666666667</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1068,6 +1107,9 @@
       <c r="M13" s="3" t="n">
         <v>0.09256</v>
       </c>
+      <c r="N13" s="3" t="n">
+        <v>0.09256</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1113,6 +1155,9 @@
       <c r="M14" s="3" t="n">
         <v>0.093975</v>
       </c>
+      <c r="N14" s="3" t="n">
+        <v>0.093975</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1158,6 +1203,9 @@
       <c r="M15" s="3" t="n">
         <v>0.094675</v>
       </c>
+      <c r="N15" s="3" t="n">
+        <v>0.09461249999999999</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1203,6 +1251,9 @@
       <c r="M16" s="3" t="n">
         <v>0.09549999999999999</v>
       </c>
+      <c r="N16" s="3" t="n">
+        <v>0.09549999999999999</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1248,6 +1299,9 @@
       <c r="M17" s="3" t="n">
         <v>0.09602500000000001</v>
       </c>
+      <c r="N17" s="3" t="n">
+        <v>0.09606250000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1293,6 +1347,9 @@
       <c r="M18" s="3" t="n">
         <v>0.09581666666666666</v>
       </c>
+      <c r="N18" s="3" t="n">
+        <v>0.09581666666666666</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1338,6 +1395,9 @@
       <c r="M19" s="3" t="n">
         <v>0.0966375</v>
       </c>
+      <c r="N19" s="3" t="n">
+        <v>0.09669999999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1383,6 +1443,9 @@
       <c r="M20" s="3" t="n">
         <v>0.0969125</v>
       </c>
+      <c r="N20" s="3" t="n">
+        <v>0.0969125</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1428,6 +1491,9 @@
       <c r="M21" s="3" t="n">
         <v>0.0968</v>
       </c>
+      <c r="N21" s="3" t="n">
+        <v>0.0968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1473,6 +1539,9 @@
       <c r="M22" s="3" t="n">
         <v>0.09714</v>
       </c>
+      <c r="N22" s="3" t="n">
+        <v>0.09714</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1518,6 +1587,9 @@
       <c r="M23" s="3" t="n">
         <v>0.09820000000000001</v>
       </c>
+      <c r="N23" s="3" t="n">
+        <v>0.0984</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1563,6 +1635,9 @@
       <c r="M24" s="3" t="n">
         <v>0.09758</v>
       </c>
+      <c r="N24" s="3" t="n">
+        <v>0.09758</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1608,6 +1683,9 @@
       <c r="M25" s="3" t="n">
         <v>0.0987625</v>
       </c>
+      <c r="N25" s="3" t="n">
+        <v>0.09884999999999999</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1653,6 +1731,9 @@
       <c r="M26" s="3" t="n">
         <v>0.09889999999999999</v>
       </c>
+      <c r="N26" s="3" t="n">
+        <v>0.09889999999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1698,6 +1779,9 @@
       <c r="M27" s="3" t="n">
         <v>0.09940000000000002</v>
       </c>
+      <c r="N27" s="3" t="n">
+        <v>0.09945555555555557</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1743,6 +1827,9 @@
       <c r="M28" s="3" t="n">
         <v>0.09975000000000001</v>
       </c>
+      <c r="N28" s="3" t="n">
+        <v>0.0996875</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1788,6 +1875,9 @@
       <c r="M29" s="3" t="n">
         <v>0.09975000000000001</v>
       </c>
+      <c r="N29" s="3" t="n">
+        <v>0.09975000000000001</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1833,6 +1923,9 @@
       <c r="M30" s="3" t="n">
         <v>0.1003428571428572</v>
       </c>
+      <c r="N30" s="3" t="n">
+        <v>0.1003428571428572</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1878,6 +1971,9 @@
       <c r="M31" s="3" t="n">
         <v>0.10045</v>
       </c>
+      <c r="N31" s="3" t="n">
+        <v>0.10045</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1923,6 +2019,9 @@
       <c r="M32" s="3" t="n">
         <v>0.1012857142857143</v>
       </c>
+      <c r="N32" s="3" t="n">
+        <v>0.1014375</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1968,6 +2067,9 @@
       <c r="M33" s="3" t="n">
         <v>0.1011</v>
       </c>
+      <c r="N33" s="3" t="n">
+        <v>0.1011</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2013,6 +2115,9 @@
       <c r="M34" s="3" t="n">
         <v>0.1016</v>
       </c>
+      <c r="N34" s="3" t="n">
+        <v>0.1016</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2058,6 +2163,9 @@
       <c r="M35" s="3" t="n">
         <v>0.1032</v>
       </c>
+      <c r="N35" s="3" t="n">
+        <v>0.1032</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2103,6 +2211,9 @@
       <c r="M36" s="3" t="n">
         <v>0.1053333333333333</v>
       </c>
+      <c r="N36" s="3" t="n">
+        <v>0.1053333333333333</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2148,6 +2259,9 @@
       <c r="M37" s="3" t="n">
         <v>0.106225</v>
       </c>
+      <c r="N37" s="3" t="n">
+        <v>0.1062875</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2193,6 +2307,9 @@
       <c r="M38" s="3" t="n">
         <v>0.1068444444444445</v>
       </c>
+      <c r="N38" s="3" t="n">
+        <v>0.1069555555555556</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2238,6 +2355,9 @@
       <c r="M39" s="3" t="n">
         <v>0.10728</v>
       </c>
+      <c r="N39" s="3" t="n">
+        <v>0.10728</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2283,6 +2403,9 @@
       <c r="M40" s="3" t="n">
         <v>0.1089666666666667</v>
       </c>
+      <c r="N40" s="3" t="n">
+        <v>0.1090444444444444</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2328,6 +2451,9 @@
       <c r="M41" s="3" t="n">
         <v>0.1082</v>
       </c>
+      <c r="N41" s="3" t="n">
+        <v>0.1082</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2373,6 +2499,9 @@
       <c r="M42" s="3" t="n">
         <v>0.1090375</v>
       </c>
+      <c r="N42" s="3" t="n">
+        <v>0.1090375</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2418,6 +2547,9 @@
       <c r="M43" s="3" t="n">
         <v>0.10912</v>
       </c>
+      <c r="N43" s="3" t="n">
+        <v>0.10912</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2463,6 +2595,9 @@
       <c r="M44" s="3" t="n">
         <v>0.1104444444444445</v>
       </c>
+      <c r="N44" s="3" t="n">
+        <v>0.1105</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2508,6 +2643,9 @@
       <c r="M45" s="3" t="n">
         <v>0.1102285714285714</v>
       </c>
+      <c r="N45" s="3" t="n">
+        <v>0.1102285714285714</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2553,6 +2691,9 @@
       <c r="M46" s="3" t="n">
         <v>0.11</v>
       </c>
+      <c r="N46" s="3" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2598,6 +2739,9 @@
       <c r="M47" s="3" t="n">
         <v>0.1107714285714286</v>
       </c>
+      <c r="N47" s="3" t="n">
+        <v>0.11095</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2643,6 +2787,9 @@
       <c r="M48" s="3" t="n">
         <v>0.1106</v>
       </c>
+      <c r="N48" s="3" t="n">
+        <v>0.1106</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2688,6 +2835,9 @@
       <c r="M49" s="3" t="n">
         <v>0.1115714285714286</v>
       </c>
+      <c r="N49" s="3" t="n">
+        <v>0.1115714285714286</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2733,6 +2883,9 @@
       <c r="M50" s="3" t="n">
         <v>0.1117</v>
       </c>
+      <c r="N50" s="3" t="n">
+        <v>0.1117</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2778,6 +2931,9 @@
       <c r="M51" s="3" t="n">
         <v>0.112625</v>
       </c>
+      <c r="N51" s="3" t="n">
+        <v>0.112625</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2823,6 +2979,9 @@
       <c r="M52" s="3" t="n">
         <v>0.1135</v>
       </c>
+      <c r="N52" s="3" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2868,6 +3027,9 @@
       <c r="M53" s="3" t="n">
         <v>0.114</v>
       </c>
+      <c r="N53" s="3" t="n">
+        <v>0.114</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2913,6 +3075,9 @@
       <c r="M54" s="3" t="n">
         <v>0.1145</v>
       </c>
+      <c r="N54" s="3" t="n">
+        <v>0.1145</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2956,6 +3121,9 @@
         <v>0.1165</v>
       </c>
       <c r="M55" s="3" t="n">
+        <v>0.1165</v>
+      </c>
+      <c r="N55" s="3" t="n">
         <v>0.1165</v>
       </c>
     </row>
@@ -2970,7 +3138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2986,6 +3154,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3054,6 +3223,11 @@
           <t>22-Apr-26</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>23-Apr-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3099,6 +3273,9 @@
       <c r="M2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3144,6 +3321,9 @@
       <c r="M3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="N3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3189,6 +3369,9 @@
       <c r="M4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3234,6 +3417,9 @@
       <c r="M5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="N5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3279,6 +3465,9 @@
       <c r="M6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3324,6 +3513,9 @@
       <c r="M7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3369,6 +3561,9 @@
       <c r="M8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3414,6 +3609,9 @@
       <c r="M9" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N9" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3459,6 +3657,9 @@
       <c r="M10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3504,6 +3705,9 @@
       <c r="M11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3549,6 +3753,9 @@
       <c r="M12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3594,6 +3801,9 @@
       <c r="M13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3639,6 +3849,9 @@
       <c r="M14" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N14" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3684,6 +3897,9 @@
       <c r="M15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3729,6 +3945,9 @@
       <c r="M16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3774,6 +3993,9 @@
       <c r="M17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3819,6 +4041,9 @@
       <c r="M18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3864,6 +4089,9 @@
       <c r="M19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3909,6 +4137,9 @@
       <c r="M20" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N20" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3954,6 +4185,9 @@
       <c r="M21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3999,6 +4233,9 @@
       <c r="M22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4044,6 +4281,9 @@
       <c r="M23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4089,6 +4329,9 @@
       <c r="M24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4134,6 +4377,9 @@
       <c r="M25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4179,6 +4425,9 @@
       <c r="M26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4224,6 +4473,9 @@
       <c r="M27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4269,6 +4521,9 @@
       <c r="M28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4314,6 +4569,9 @@
       <c r="M29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4359,6 +4617,9 @@
       <c r="M30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4404,6 +4665,9 @@
       <c r="M31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4449,6 +4713,9 @@
       <c r="M32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4494,6 +4761,9 @@
       <c r="M33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4539,6 +4809,9 @@
       <c r="M34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4584,6 +4857,9 @@
       <c r="M35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4629,6 +4905,9 @@
       <c r="M36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4674,6 +4953,9 @@
       <c r="M37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4719,6 +5001,9 @@
       <c r="M38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4764,6 +5049,9 @@
       <c r="M39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="N39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4807,6 +5095,9 @@
         <v>0.13</v>
       </c>
       <c r="M40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="N40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update treasury bond yields - 2026-04-29
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:O55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -461,6 +461,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,6 +535,11 @@
           <t>23-Apr-26</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>28-Apr-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -582,6 +588,9 @@
       <c r="N2" s="3" t="n">
         <v>0.08153333333333335</v>
       </c>
+      <c r="O2" s="3" t="n">
+        <v>0.08145000000000001</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -630,6 +639,9 @@
       <c r="N3" s="3" t="n">
         <v>0.08188333333333335</v>
       </c>
+      <c r="O3" s="3" t="n">
+        <v>0.08180000000000001</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -678,6 +690,9 @@
       <c r="N4" s="3" t="n">
         <v>0.08297142857142858</v>
       </c>
+      <c r="O4" s="3" t="n">
+        <v>0.08299999999999999</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -726,6 +741,9 @@
       <c r="N5" s="3" t="n">
         <v>0.08493333333333335</v>
       </c>
+      <c r="O5" s="3" t="n">
+        <v>0.08510000000000001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -774,6 +792,9 @@
       <c r="N6" s="3" t="n">
         <v>0.08473333333333333</v>
       </c>
+      <c r="O6" s="3" t="n">
+        <v>0.08506666666666667</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -822,6 +843,9 @@
       <c r="N7" s="3" t="n">
         <v>0.08664285714285715</v>
       </c>
+      <c r="O7" s="3" t="n">
+        <v>0.08642857142857142</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -870,6 +894,9 @@
       <c r="N8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="O8" s="3" t="n">
+        <v>0.08629999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -918,6 +945,9 @@
       <c r="N9" s="3" t="n">
         <v>0.08851999999999999</v>
       </c>
+      <c r="O9" s="3" t="n">
+        <v>0.08851999999999999</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -966,6 +996,9 @@
       <c r="N10" s="3" t="n">
         <v>0.08972857142857142</v>
       </c>
+      <c r="O10" s="3" t="n">
+        <v>0.0898875</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1014,6 +1047,9 @@
       <c r="N11" s="3" t="n">
         <v>0.08984</v>
       </c>
+      <c r="O11" s="3" t="n">
+        <v>0.08984</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1062,6 +1098,9 @@
       <c r="N12" s="3" t="n">
         <v>0.09111666666666667</v>
       </c>
+      <c r="O12" s="3" t="n">
+        <v>0.09111666666666667</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1110,6 +1149,9 @@
       <c r="N13" s="3" t="n">
         <v>0.09256</v>
       </c>
+      <c r="O13" s="3" t="n">
+        <v>0.09265999999999999</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1158,6 +1200,9 @@
       <c r="N14" s="3" t="n">
         <v>0.093975</v>
       </c>
+      <c r="O14" s="3" t="n">
+        <v>0.09447777777777777</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1206,6 +1251,9 @@
       <c r="N15" s="3" t="n">
         <v>0.09461249999999999</v>
       </c>
+      <c r="O15" s="3" t="n">
+        <v>0.09462857142857141</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1254,6 +1302,9 @@
       <c r="N16" s="3" t="n">
         <v>0.09549999999999999</v>
       </c>
+      <c r="O16" s="3" t="n">
+        <v>0.09543749999999999</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1302,6 +1353,9 @@
       <c r="N17" s="3" t="n">
         <v>0.09606250000000001</v>
       </c>
+      <c r="O17" s="3" t="n">
+        <v>0.09615</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1350,6 +1404,9 @@
       <c r="N18" s="3" t="n">
         <v>0.09581666666666666</v>
       </c>
+      <c r="O18" s="3" t="n">
+        <v>0.09598333333333332</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1398,6 +1455,9 @@
       <c r="N19" s="3" t="n">
         <v>0.09669999999999999</v>
       </c>
+      <c r="O19" s="3" t="n">
+        <v>0.09694999999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1446,6 +1506,9 @@
       <c r="N20" s="3" t="n">
         <v>0.0969125</v>
       </c>
+      <c r="O20" s="3" t="n">
+        <v>0.09736666666666666</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1494,6 +1557,9 @@
       <c r="N21" s="3" t="n">
         <v>0.0968</v>
       </c>
+      <c r="O21" s="3" t="n">
+        <v>0.0968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1542,6 +1608,9 @@
       <c r="N22" s="3" t="n">
         <v>0.09714</v>
       </c>
+      <c r="O22" s="3" t="n">
+        <v>0.09714</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1590,6 +1659,9 @@
       <c r="N23" s="3" t="n">
         <v>0.0984</v>
       </c>
+      <c r="O23" s="3" t="n">
+        <v>0.09853333333333333</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1638,6 +1710,9 @@
       <c r="N24" s="3" t="n">
         <v>0.09758</v>
       </c>
+      <c r="O24" s="3" t="n">
+        <v>0.09758</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1686,6 +1761,9 @@
       <c r="N25" s="3" t="n">
         <v>0.09884999999999999</v>
       </c>
+      <c r="O25" s="3" t="n">
+        <v>0.0987875</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1734,6 +1812,9 @@
       <c r="N26" s="3" t="n">
         <v>0.09889999999999999</v>
       </c>
+      <c r="O26" s="3" t="n">
+        <v>0.09889999999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1782,6 +1863,9 @@
       <c r="N27" s="3" t="n">
         <v>0.09945555555555557</v>
       </c>
+      <c r="O27" s="3" t="n">
+        <v>0.09951111111111112</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1830,6 +1914,9 @@
       <c r="N28" s="3" t="n">
         <v>0.0996875</v>
       </c>
+      <c r="O28" s="3" t="n">
+        <v>0.09975000000000001</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1878,6 +1965,9 @@
       <c r="N29" s="3" t="n">
         <v>0.09975000000000001</v>
       </c>
+      <c r="O29" s="3" t="n">
+        <v>0.09983333333333333</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1926,6 +2016,9 @@
       <c r="N30" s="3" t="n">
         <v>0.1003428571428572</v>
       </c>
+      <c r="O30" s="3" t="n">
+        <v>0.1003428571428572</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1974,6 +2067,9 @@
       <c r="N31" s="3" t="n">
         <v>0.10045</v>
       </c>
+      <c r="O31" s="3" t="n">
+        <v>0.10045</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2022,6 +2118,9 @@
       <c r="N32" s="3" t="n">
         <v>0.1014375</v>
       </c>
+      <c r="O32" s="3" t="n">
+        <v>0.101375</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2070,6 +2169,9 @@
       <c r="N33" s="3" t="n">
         <v>0.1011</v>
       </c>
+      <c r="O33" s="3" t="n">
+        <v>0.1011</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2118,6 +2220,9 @@
       <c r="N34" s="3" t="n">
         <v>0.1016</v>
       </c>
+      <c r="O34" s="3" t="n">
+        <v>0.1016</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2166,6 +2271,9 @@
       <c r="N35" s="3" t="n">
         <v>0.1032</v>
       </c>
+      <c r="O35" s="3" t="n">
+        <v>0.1032</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2214,6 +2322,9 @@
       <c r="N36" s="3" t="n">
         <v>0.1053333333333333</v>
       </c>
+      <c r="O36" s="3" t="n">
+        <v>0.1053333333333333</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2262,6 +2373,9 @@
       <c r="N37" s="3" t="n">
         <v>0.1062875</v>
       </c>
+      <c r="O37" s="3" t="n">
+        <v>0.1061625</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2310,6 +2424,9 @@
       <c r="N38" s="3" t="n">
         <v>0.1069555555555556</v>
       </c>
+      <c r="O38" s="3" t="n">
+        <v>0.10716</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2358,6 +2475,9 @@
       <c r="N39" s="3" t="n">
         <v>0.10728</v>
       </c>
+      <c r="O39" s="3" t="n">
+        <v>0.10728</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2406,6 +2526,9 @@
       <c r="N40" s="3" t="n">
         <v>0.1090444444444444</v>
       </c>
+      <c r="O40" s="3" t="n">
+        <v>0.1090222222222222</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2454,6 +2577,9 @@
       <c r="N41" s="3" t="n">
         <v>0.1082</v>
       </c>
+      <c r="O41" s="3" t="n">
+        <v>0.1082</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2502,6 +2628,9 @@
       <c r="N42" s="3" t="n">
         <v>0.1090375</v>
       </c>
+      <c r="O42" s="3" t="n">
+        <v>0.1090375</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2550,6 +2679,9 @@
       <c r="N43" s="3" t="n">
         <v>0.10912</v>
       </c>
+      <c r="O43" s="3" t="n">
+        <v>0.10912</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2598,6 +2730,9 @@
       <c r="N44" s="3" t="n">
         <v>0.1105</v>
       </c>
+      <c r="O44" s="3" t="n">
+        <v>0.1105333333333333</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2646,6 +2781,9 @@
       <c r="N45" s="3" t="n">
         <v>0.1102285714285714</v>
       </c>
+      <c r="O45" s="3" t="n">
+        <v>0.1099833333333333</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2694,6 +2832,9 @@
       <c r="N46" s="3" t="n">
         <v>0.11</v>
       </c>
+      <c r="O46" s="3" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2742,6 +2883,9 @@
       <c r="N47" s="3" t="n">
         <v>0.11095</v>
       </c>
+      <c r="O47" s="3" t="n">
+        <v>0.11095</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2790,6 +2934,9 @@
       <c r="N48" s="3" t="n">
         <v>0.1106</v>
       </c>
+      <c r="O48" s="3" t="n">
+        <v>0.1106</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2838,6 +2985,9 @@
       <c r="N49" s="3" t="n">
         <v>0.1115714285714286</v>
       </c>
+      <c r="O49" s="3" t="n">
+        <v>0.1112833333333333</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2886,6 +3036,9 @@
       <c r="N50" s="3" t="n">
         <v>0.1117</v>
       </c>
+      <c r="O50" s="3" t="n">
+        <v>0.1116</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2934,6 +3087,9 @@
       <c r="N51" s="3" t="n">
         <v>0.112625</v>
       </c>
+      <c r="O51" s="3" t="n">
+        <v>0.112625</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2982,6 +3138,9 @@
       <c r="N52" s="3" t="n">
         <v>0.1135</v>
       </c>
+      <c r="O52" s="3" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3030,6 +3189,9 @@
       <c r="N53" s="3" t="n">
         <v>0.114</v>
       </c>
+      <c r="O53" s="3" t="n">
+        <v>0.114</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3078,6 +3240,9 @@
       <c r="N54" s="3" t="n">
         <v>0.1145</v>
       </c>
+      <c r="O54" s="3" t="n">
+        <v>0.1145</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3124,6 +3289,9 @@
         <v>0.1165</v>
       </c>
       <c r="N55" s="3" t="n">
+        <v>0.1165</v>
+      </c>
+      <c r="O55" s="3" t="n">
         <v>0.1165</v>
       </c>
     </row>
@@ -3138,7 +3306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3155,6 +3323,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3228,6 +3397,11 @@
           <t>23-Apr-26</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>28-Apr-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3276,6 +3450,9 @@
       <c r="N2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3324,6 +3501,9 @@
       <c r="N3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="O3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3372,6 +3552,9 @@
       <c r="N4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3420,6 +3603,9 @@
       <c r="N5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="O5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3468,6 +3654,9 @@
       <c r="N6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3516,6 +3705,9 @@
       <c r="N7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3564,6 +3756,9 @@
       <c r="N8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3612,6 +3807,9 @@
       <c r="N9" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O9" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3660,6 +3858,9 @@
       <c r="N10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3708,6 +3909,9 @@
       <c r="N11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3756,6 +3960,9 @@
       <c r="N12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3804,6 +4011,9 @@
       <c r="N13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3852,6 +4062,9 @@
       <c r="N14" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O14" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3900,6 +4113,9 @@
       <c r="N15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3948,6 +4164,9 @@
       <c r="N16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3996,6 +4215,9 @@
       <c r="N17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4044,6 +4266,9 @@
       <c r="N18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4092,6 +4317,9 @@
       <c r="N19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4140,6 +4368,9 @@
       <c r="N20" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O20" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4188,6 +4419,9 @@
       <c r="N21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4236,6 +4470,9 @@
       <c r="N22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4284,6 +4521,9 @@
       <c r="N23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4332,6 +4572,9 @@
       <c r="N24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4380,6 +4623,9 @@
       <c r="N25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4428,6 +4674,9 @@
       <c r="N26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4476,6 +4725,9 @@
       <c r="N27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4524,6 +4776,9 @@
       <c r="N28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4572,6 +4827,9 @@
       <c r="N29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4620,6 +4878,9 @@
       <c r="N30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4668,6 +4929,9 @@
       <c r="N31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4716,6 +4980,9 @@
       <c r="N32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4764,6 +5031,9 @@
       <c r="N33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4812,6 +5082,9 @@
       <c r="N34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4860,6 +5133,9 @@
       <c r="N35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4908,6 +5184,9 @@
       <c r="N36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4956,6 +5235,9 @@
       <c r="N37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5004,6 +5286,9 @@
       <c r="N38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5052,6 +5337,9 @@
       <c r="N39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="O39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5098,6 +5386,9 @@
         <v>0.13</v>
       </c>
       <c r="N40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="O40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update treasury bond yields - 2026-04-30
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -462,6 +462,7 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,6 +541,11 @@
           <t>28-Apr-26</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>29-Apr-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -591,6 +597,9 @@
       <c r="O2" s="3" t="n">
         <v>0.08145000000000001</v>
       </c>
+      <c r="P2" s="3" t="n">
+        <v>0.08136666666666668</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -642,6 +651,9 @@
       <c r="O3" s="3" t="n">
         <v>0.08180000000000001</v>
       </c>
+      <c r="P3" s="3" t="n">
+        <v>0.0818</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -693,6 +705,9 @@
       <c r="O4" s="3" t="n">
         <v>0.08299999999999999</v>
       </c>
+      <c r="P4" s="3" t="n">
+        <v>0.08291249999999999</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -744,6 +759,9 @@
       <c r="O5" s="3" t="n">
         <v>0.08510000000000001</v>
       </c>
+      <c r="P5" s="3" t="n">
+        <v>0.08498888888888891</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -795,6 +813,9 @@
       <c r="O6" s="3" t="n">
         <v>0.08506666666666667</v>
       </c>
+      <c r="P6" s="3" t="n">
+        <v>0.08427999999999999</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -846,6 +867,9 @@
       <c r="O7" s="3" t="n">
         <v>0.08642857142857142</v>
       </c>
+      <c r="P7" s="3" t="n">
+        <v>0.08624285714285716</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -897,6 +921,9 @@
       <c r="O8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="P8" s="3" t="n">
+        <v>0.08629999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -948,6 +975,9 @@
       <c r="O9" s="3" t="n">
         <v>0.08851999999999999</v>
       </c>
+      <c r="P9" s="3" t="n">
+        <v>0.08851999999999999</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -999,6 +1029,9 @@
       <c r="O10" s="3" t="n">
         <v>0.0898875</v>
       </c>
+      <c r="P10" s="3" t="n">
+        <v>0.08995</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1050,6 +1083,9 @@
       <c r="O11" s="3" t="n">
         <v>0.08984</v>
       </c>
+      <c r="P11" s="3" t="n">
+        <v>0.08984</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1101,6 +1137,9 @@
       <c r="O12" s="3" t="n">
         <v>0.09111666666666667</v>
       </c>
+      <c r="P12" s="3" t="n">
+        <v>0.09111666666666667</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1152,6 +1191,9 @@
       <c r="O13" s="3" t="n">
         <v>0.09265999999999999</v>
       </c>
+      <c r="P13" s="3" t="n">
+        <v>0.09304999999999998</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1203,6 +1245,9 @@
       <c r="O14" s="3" t="n">
         <v>0.09447777777777777</v>
       </c>
+      <c r="P14" s="3" t="n">
+        <v>0.09442222222222221</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1254,6 +1299,9 @@
       <c r="O15" s="3" t="n">
         <v>0.09462857142857141</v>
       </c>
+      <c r="P15" s="3" t="n">
+        <v>0.09462857142857141</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1305,6 +1353,9 @@
       <c r="O16" s="3" t="n">
         <v>0.09543749999999999</v>
       </c>
+      <c r="P16" s="3" t="n">
+        <v>0.095375</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1356,6 +1407,9 @@
       <c r="O17" s="3" t="n">
         <v>0.09615</v>
       </c>
+      <c r="P17" s="3" t="n">
+        <v>0.09608750000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1407,6 +1461,9 @@
       <c r="O18" s="3" t="n">
         <v>0.09598333333333332</v>
       </c>
+      <c r="P18" s="3" t="n">
+        <v>0.09619999999999998</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1458,6 +1515,9 @@
       <c r="O19" s="3" t="n">
         <v>0.09694999999999999</v>
       </c>
+      <c r="P19" s="3" t="n">
+        <v>0.09663749999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1509,6 +1569,9 @@
       <c r="O20" s="3" t="n">
         <v>0.09736666666666666</v>
       </c>
+      <c r="P20" s="3" t="n">
+        <v>0.097</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1560,6 +1623,9 @@
       <c r="O21" s="3" t="n">
         <v>0.0968</v>
       </c>
+      <c r="P21" s="3" t="n">
+        <v>0.0968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1611,6 +1677,9 @@
       <c r="O22" s="3" t="n">
         <v>0.09714</v>
       </c>
+      <c r="P22" s="3" t="n">
+        <v>0.09714</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1662,6 +1731,9 @@
       <c r="O23" s="3" t="n">
         <v>0.09853333333333333</v>
       </c>
+      <c r="P23" s="3" t="n">
+        <v>0.09825555555555557</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1713,6 +1785,9 @@
       <c r="O24" s="3" t="n">
         <v>0.09758</v>
       </c>
+      <c r="P24" s="3" t="n">
+        <v>0.09815</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1764,6 +1839,9 @@
       <c r="O25" s="3" t="n">
         <v>0.0987875</v>
       </c>
+      <c r="P25" s="3" t="n">
+        <v>0.0987875</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1815,6 +1893,9 @@
       <c r="O26" s="3" t="n">
         <v>0.09889999999999999</v>
       </c>
+      <c r="P26" s="3" t="n">
+        <v>0.09902499999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1866,6 +1947,9 @@
       <c r="O27" s="3" t="n">
         <v>0.09951111111111112</v>
       </c>
+      <c r="P27" s="3" t="n">
+        <v>0.09953333333333333</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1917,6 +2001,9 @@
       <c r="O28" s="3" t="n">
         <v>0.09975000000000001</v>
       </c>
+      <c r="P28" s="3" t="n">
+        <v>0.09981250000000001</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1968,6 +2055,9 @@
       <c r="O29" s="3" t="n">
         <v>0.09983333333333333</v>
       </c>
+      <c r="P29" s="3" t="n">
+        <v>0.1000833333333333</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2019,6 +2109,9 @@
       <c r="O30" s="3" t="n">
         <v>0.1003428571428572</v>
       </c>
+      <c r="P30" s="3" t="n">
+        <v>0.1005571428571429</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2070,6 +2163,9 @@
       <c r="O31" s="3" t="n">
         <v>0.10045</v>
       </c>
+      <c r="P31" s="3" t="n">
+        <v>0.1007</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2121,6 +2217,9 @@
       <c r="O32" s="3" t="n">
         <v>0.101375</v>
       </c>
+      <c r="P32" s="3" t="n">
+        <v>0.1015625</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2172,6 +2271,9 @@
       <c r="O33" s="3" t="n">
         <v>0.1011</v>
       </c>
+      <c r="P33" s="3" t="n">
+        <v>0.1018333333333333</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2223,6 +2325,9 @@
       <c r="O34" s="3" t="n">
         <v>0.1016</v>
       </c>
+      <c r="P34" s="3" t="n">
+        <v>0.1023333333333333</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2274,6 +2379,9 @@
       <c r="O35" s="3" t="n">
         <v>0.1032</v>
       </c>
+      <c r="P35" s="3" t="n">
+        <v>0.1044</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2325,6 +2433,9 @@
       <c r="O36" s="3" t="n">
         <v>0.1053333333333333</v>
       </c>
+      <c r="P36" s="3" t="n">
+        <v>0.1058333333333333</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2376,6 +2487,9 @@
       <c r="O37" s="3" t="n">
         <v>0.1061625</v>
       </c>
+      <c r="P37" s="3" t="n">
+        <v>0.1066625</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2427,6 +2541,9 @@
       <c r="O38" s="3" t="n">
         <v>0.10716</v>
       </c>
+      <c r="P38" s="3" t="n">
+        <v>0.10762</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2478,6 +2595,9 @@
       <c r="O39" s="3" t="n">
         <v>0.10728</v>
       </c>
+      <c r="P39" s="3" t="n">
+        <v>0.10798</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2529,6 +2649,9 @@
       <c r="O40" s="3" t="n">
         <v>0.1090222222222222</v>
       </c>
+      <c r="P40" s="3" t="n">
+        <v>0.1093222222222222</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2580,6 +2703,9 @@
       <c r="O41" s="3" t="n">
         <v>0.1082</v>
       </c>
+      <c r="P41" s="3" t="n">
+        <v>0.1087</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2631,6 +2757,9 @@
       <c r="O42" s="3" t="n">
         <v>0.1090375</v>
       </c>
+      <c r="P42" s="3" t="n">
+        <v>0.1094375</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2682,6 +2811,9 @@
       <c r="O43" s="3" t="n">
         <v>0.10912</v>
       </c>
+      <c r="P43" s="3" t="n">
+        <v>0.10932</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2733,6 +2865,9 @@
       <c r="O44" s="3" t="n">
         <v>0.1105333333333333</v>
       </c>
+      <c r="P44" s="3" t="n">
+        <v>0.1106777777777778</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2784,6 +2919,9 @@
       <c r="O45" s="3" t="n">
         <v>0.1099833333333333</v>
       </c>
+      <c r="P45" s="3" t="n">
+        <v>0.11015</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2835,6 +2973,9 @@
       <c r="O46" s="3" t="n">
         <v>0.11</v>
       </c>
+      <c r="P46" s="3" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2886,6 +3027,9 @@
       <c r="O47" s="3" t="n">
         <v>0.11095</v>
       </c>
+      <c r="P47" s="3" t="n">
+        <v>0.11095</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2937,6 +3081,9 @@
       <c r="O48" s="3" t="n">
         <v>0.1106</v>
       </c>
+      <c r="P48" s="3" t="n">
+        <v>0.111</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2988,6 +3135,9 @@
       <c r="O49" s="3" t="n">
         <v>0.1112833333333333</v>
       </c>
+      <c r="P49" s="3" t="n">
+        <v>0.1115285714285714</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3039,6 +3189,9 @@
       <c r="O50" s="3" t="n">
         <v>0.1116</v>
       </c>
+      <c r="P50" s="3" t="n">
+        <v>0.1116</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3090,6 +3243,9 @@
       <c r="O51" s="3" t="n">
         <v>0.112625</v>
       </c>
+      <c r="P51" s="3" t="n">
+        <v>0.112625</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3141,6 +3297,9 @@
       <c r="O52" s="3" t="n">
         <v>0.1135</v>
       </c>
+      <c r="P52" s="3" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3192,6 +3351,9 @@
       <c r="O53" s="3" t="n">
         <v>0.114</v>
       </c>
+      <c r="P53" s="3" t="n">
+        <v>0.114</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3243,6 +3405,9 @@
       <c r="O54" s="3" t="n">
         <v>0.1145</v>
       </c>
+      <c r="P54" s="3" t="n">
+        <v>0.1145</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3292,6 +3457,9 @@
         <v>0.1165</v>
       </c>
       <c r="O55" s="3" t="n">
+        <v>0.1165</v>
+      </c>
+      <c r="P55" s="3" t="n">
         <v>0.1165</v>
       </c>
     </row>
@@ -3306,7 +3474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O40"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3324,6 +3492,7 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3402,6 +3571,11 @@
           <t>28-Apr-26</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>29-Apr-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3453,6 +3627,9 @@
       <c r="O2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3504,6 +3681,9 @@
       <c r="O3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="P3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3555,6 +3735,9 @@
       <c r="O4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3606,6 +3789,9 @@
       <c r="O5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="P5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3657,6 +3843,9 @@
       <c r="O6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3708,6 +3897,9 @@
       <c r="O7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3759,6 +3951,9 @@
       <c r="O8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3810,6 +4005,9 @@
       <c r="O9" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P9" s="3" t="n">
+        <v>0.1444</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3861,6 +4059,9 @@
       <c r="O10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3912,6 +4113,9 @@
       <c r="O11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3963,6 +4167,9 @@
       <c r="O12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4014,6 +4221,9 @@
       <c r="O13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4065,6 +4275,9 @@
       <c r="O14" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P14" s="3" t="n">
+        <v>0.1454</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4116,6 +4329,9 @@
       <c r="O15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4167,6 +4383,9 @@
       <c r="O16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4218,6 +4437,9 @@
       <c r="O17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4269,6 +4491,9 @@
       <c r="O18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4320,6 +4545,9 @@
       <c r="O19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4371,6 +4599,9 @@
       <c r="O20" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P20" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4422,6 +4653,9 @@
       <c r="O21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4473,6 +4707,9 @@
       <c r="O22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4524,6 +4761,9 @@
       <c r="O23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4575,6 +4815,9 @@
       <c r="O24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4626,6 +4869,9 @@
       <c r="O25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4677,6 +4923,9 @@
       <c r="O26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4728,6 +4977,9 @@
       <c r="O27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4779,6 +5031,9 @@
       <c r="O28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4830,6 +5085,9 @@
       <c r="O29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4881,6 +5139,9 @@
       <c r="O30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4932,6 +5193,9 @@
       <c r="O31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4983,6 +5247,9 @@
       <c r="O32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5034,6 +5301,9 @@
       <c r="O33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5085,6 +5355,9 @@
       <c r="O34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5136,6 +5409,9 @@
       <c r="O35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5187,6 +5463,9 @@
       <c r="O36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5238,6 +5517,9 @@
       <c r="O37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5289,6 +5571,9 @@
       <c r="O38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5340,6 +5625,9 @@
       <c r="O39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="P39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5389,6 +5677,9 @@
         <v>0.13</v>
       </c>
       <c r="O40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="P40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update treasury bond yields - 2026-05-06
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P55"/>
+  <dimension ref="A1:Q55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -463,6 +463,7 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,6 +547,11 @@
           <t>29-Apr-26</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>06-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -600,6 +606,9 @@
       <c r="P2" s="3" t="n">
         <v>0.08136666666666668</v>
       </c>
+      <c r="Q2" s="3" t="n">
+        <v>0.08136666666666668</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -654,6 +663,9 @@
       <c r="P3" s="3" t="n">
         <v>0.0818</v>
       </c>
+      <c r="Q3" s="3" t="n">
+        <v>0.0818</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -708,6 +720,9 @@
       <c r="P4" s="3" t="n">
         <v>0.08291249999999999</v>
       </c>
+      <c r="Q4" s="3" t="n">
+        <v>0.08318571428571429</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -762,6 +777,9 @@
       <c r="P5" s="3" t="n">
         <v>0.08498888888888891</v>
       </c>
+      <c r="Q5" s="3" t="n">
+        <v>0.08448750000000001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -816,6 +834,9 @@
       <c r="P6" s="3" t="n">
         <v>0.08427999999999999</v>
       </c>
+      <c r="Q6" s="3" t="n">
+        <v>0.08427999999999999</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -870,6 +891,9 @@
       <c r="P7" s="3" t="n">
         <v>0.08624285714285716</v>
       </c>
+      <c r="Q7" s="3" t="n">
+        <v>0.08650000000000001</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -924,6 +948,9 @@
       <c r="P8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="Q8" s="3" t="n">
+        <v>0.08629999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -978,6 +1005,9 @@
       <c r="P9" s="3" t="n">
         <v>0.08851999999999999</v>
       </c>
+      <c r="Q9" s="3" t="n">
+        <v>0.08851999999999999</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1032,6 +1062,9 @@
       <c r="P10" s="3" t="n">
         <v>0.08995</v>
       </c>
+      <c r="Q10" s="3" t="n">
+        <v>0.0901375</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1086,6 +1119,9 @@
       <c r="P11" s="3" t="n">
         <v>0.08984</v>
       </c>
+      <c r="Q11" s="3" t="n">
+        <v>0.08984</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1140,6 +1176,9 @@
       <c r="P12" s="3" t="n">
         <v>0.09111666666666667</v>
       </c>
+      <c r="Q12" s="3" t="n">
+        <v>0.09111666666666667</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1194,6 +1233,9 @@
       <c r="P13" s="3" t="n">
         <v>0.09304999999999998</v>
       </c>
+      <c r="Q13" s="3" t="n">
+        <v>0.09304999999999998</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1248,6 +1290,9 @@
       <c r="P14" s="3" t="n">
         <v>0.09442222222222221</v>
       </c>
+      <c r="Q14" s="3" t="n">
+        <v>0.09497777777777777</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1302,6 +1347,9 @@
       <c r="P15" s="3" t="n">
         <v>0.09462857142857141</v>
       </c>
+      <c r="Q15" s="3" t="n">
+        <v>0.09484285714285713</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1356,6 +1404,9 @@
       <c r="P16" s="3" t="n">
         <v>0.095375</v>
       </c>
+      <c r="Q16" s="3" t="n">
+        <v>0.096</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1410,6 +1461,9 @@
       <c r="P17" s="3" t="n">
         <v>0.09608750000000001</v>
       </c>
+      <c r="Q17" s="3" t="n">
+        <v>0.09646250000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1464,6 +1518,9 @@
       <c r="P18" s="3" t="n">
         <v>0.09619999999999998</v>
       </c>
+      <c r="Q18" s="3" t="n">
+        <v>0.09648571428571427</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1518,6 +1575,9 @@
       <c r="P19" s="3" t="n">
         <v>0.09663749999999999</v>
       </c>
+      <c r="Q19" s="3" t="n">
+        <v>0.09701249999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1572,6 +1632,9 @@
       <c r="P20" s="3" t="n">
         <v>0.097</v>
       </c>
+      <c r="Q20" s="3" t="n">
+        <v>0.09758888888888889</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1626,6 +1689,9 @@
       <c r="P21" s="3" t="n">
         <v>0.0968</v>
       </c>
+      <c r="Q21" s="3" t="n">
+        <v>0.0968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1680,6 +1746,9 @@
       <c r="P22" s="3" t="n">
         <v>0.09714</v>
       </c>
+      <c r="Q22" s="3" t="n">
+        <v>0.09778333333333333</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1734,6 +1803,9 @@
       <c r="P23" s="3" t="n">
         <v>0.09825555555555557</v>
       </c>
+      <c r="Q23" s="3" t="n">
+        <v>0.09895555555555556</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1788,6 +1860,9 @@
       <c r="P24" s="3" t="n">
         <v>0.09815</v>
       </c>
+      <c r="Q24" s="3" t="n">
+        <v>0.09758</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1842,6 +1917,9 @@
       <c r="P25" s="3" t="n">
         <v>0.0987875</v>
       </c>
+      <c r="Q25" s="3" t="n">
+        <v>0.09928750000000001</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1896,6 +1974,9 @@
       <c r="P26" s="3" t="n">
         <v>0.09902499999999999</v>
       </c>
+      <c r="Q26" s="3" t="n">
+        <v>0.09958750000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1950,6 +2031,9 @@
       <c r="P27" s="3" t="n">
         <v>0.09953333333333333</v>
       </c>
+      <c r="Q27" s="3" t="n">
+        <v>0.1000666666666667</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2004,6 +2088,9 @@
       <c r="P28" s="3" t="n">
         <v>0.09981250000000001</v>
       </c>
+      <c r="Q28" s="3" t="n">
+        <v>0.100375</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2058,6 +2145,9 @@
       <c r="P29" s="3" t="n">
         <v>0.1000833333333333</v>
       </c>
+      <c r="Q29" s="3" t="n">
+        <v>0.10025</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2112,6 +2202,9 @@
       <c r="P30" s="3" t="n">
         <v>0.1005571428571429</v>
       </c>
+      <c r="Q30" s="3" t="n">
+        <v>0.1008</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2166,6 +2259,9 @@
       <c r="P31" s="3" t="n">
         <v>0.1007</v>
       </c>
+      <c r="Q31" s="3" t="n">
+        <v>0.1008666666666667</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2220,6 +2316,9 @@
       <c r="P32" s="3" t="n">
         <v>0.1015625</v>
       </c>
+      <c r="Q32" s="3" t="n">
+        <v>0.10185</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2274,6 +2373,9 @@
       <c r="P33" s="3" t="n">
         <v>0.1018333333333333</v>
       </c>
+      <c r="Q33" s="3" t="n">
+        <v>0.1018333333333333</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2328,6 +2430,9 @@
       <c r="P34" s="3" t="n">
         <v>0.1023333333333333</v>
       </c>
+      <c r="Q34" s="3" t="n">
+        <v>0.102</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2382,6 +2487,9 @@
       <c r="P35" s="3" t="n">
         <v>0.1044</v>
       </c>
+      <c r="Q35" s="3" t="n">
+        <v>0.1043</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2436,6 +2544,9 @@
       <c r="P36" s="3" t="n">
         <v>0.1058333333333333</v>
       </c>
+      <c r="Q36" s="3" t="n">
+        <v>0.1058333333333333</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2490,6 +2601,9 @@
       <c r="P37" s="3" t="n">
         <v>0.1066625</v>
       </c>
+      <c r="Q37" s="3" t="n">
+        <v>0.10685</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2544,6 +2658,9 @@
       <c r="P38" s="3" t="n">
         <v>0.10762</v>
       </c>
+      <c r="Q38" s="3" t="n">
+        <v>0.10781</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2598,6 +2715,9 @@
       <c r="P39" s="3" t="n">
         <v>0.10798</v>
       </c>
+      <c r="Q39" s="3" t="n">
+        <v>0.10828</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2652,6 +2772,9 @@
       <c r="P40" s="3" t="n">
         <v>0.1093222222222222</v>
       </c>
+      <c r="Q40" s="3" t="n">
+        <v>0.1098555555555555</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2706,6 +2829,9 @@
       <c r="P41" s="3" t="n">
         <v>0.1087</v>
       </c>
+      <c r="Q41" s="3" t="n">
+        <v>0.10896</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2760,6 +2886,9 @@
       <c r="P42" s="3" t="n">
         <v>0.1094375</v>
       </c>
+      <c r="Q42" s="3" t="n">
+        <v>0.1099375</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2814,6 +2943,9 @@
       <c r="P43" s="3" t="n">
         <v>0.10932</v>
       </c>
+      <c r="Q43" s="3" t="n">
+        <v>0.10952</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2868,6 +3000,9 @@
       <c r="P44" s="3" t="n">
         <v>0.1106777777777778</v>
       </c>
+      <c r="Q44" s="3" t="n">
+        <v>0.110975</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2922,6 +3057,9 @@
       <c r="P45" s="3" t="n">
         <v>0.11015</v>
       </c>
+      <c r="Q45" s="3" t="n">
+        <v>0.1105333333333333</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2976,6 +3114,9 @@
       <c r="P46" s="3" t="n">
         <v>0.11</v>
       </c>
+      <c r="Q46" s="3" t="n">
+        <v>0.1101</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3030,6 +3171,9 @@
       <c r="P47" s="3" t="n">
         <v>0.11095</v>
       </c>
+      <c r="Q47" s="3" t="n">
+        <v>0.111325</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3084,6 +3228,9 @@
       <c r="P48" s="3" t="n">
         <v>0.111</v>
       </c>
+      <c r="Q48" s="3" t="n">
+        <v>0.1112166666666667</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3138,6 +3285,9 @@
       <c r="P49" s="3" t="n">
         <v>0.1115285714285714</v>
       </c>
+      <c r="Q49" s="3" t="n">
+        <v>0.1118571428571429</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3192,6 +3342,9 @@
       <c r="P50" s="3" t="n">
         <v>0.1116</v>
       </c>
+      <c r="Q50" s="3" t="n">
+        <v>0.1116</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3246,6 +3399,9 @@
       <c r="P51" s="3" t="n">
         <v>0.112625</v>
       </c>
+      <c r="Q51" s="3" t="n">
+        <v>0.112625</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3300,6 +3456,9 @@
       <c r="P52" s="3" t="n">
         <v>0.1135</v>
       </c>
+      <c r="Q52" s="3" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3354,6 +3513,9 @@
       <c r="P53" s="3" t="n">
         <v>0.114</v>
       </c>
+      <c r="Q53" s="3" t="n">
+        <v>0.114</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3408,6 +3570,9 @@
       <c r="P54" s="3" t="n">
         <v>0.1145</v>
       </c>
+      <c r="Q54" s="3" t="n">
+        <v>0.1145</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3460,6 +3625,9 @@
         <v>0.1165</v>
       </c>
       <c r="P55" s="3" t="n">
+        <v>0.1165</v>
+      </c>
+      <c r="Q55" s="3" t="n">
         <v>0.1165</v>
       </c>
     </row>
@@ -3474,7 +3642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P40"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3493,6 +3661,7 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3576,6 +3745,11 @@
           <t>29-Apr-26</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>06-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3630,6 +3804,9 @@
       <c r="P2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3684,6 +3861,9 @@
       <c r="P3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="Q3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3738,6 +3918,9 @@
       <c r="P4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3792,6 +3975,9 @@
       <c r="P5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="Q5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3846,6 +4032,9 @@
       <c r="P6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3900,6 +4089,9 @@
       <c r="P7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3954,6 +4146,9 @@
       <c r="P8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4008,6 +4203,9 @@
       <c r="P9" s="3" t="n">
         <v>0.1444</v>
       </c>
+      <c r="Q9" s="3" t="n">
+        <v>0.1444</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4062,6 +4260,9 @@
       <c r="P10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4116,6 +4317,9 @@
       <c r="P11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4170,6 +4374,9 @@
       <c r="P12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4224,6 +4431,9 @@
       <c r="P13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4278,6 +4488,9 @@
       <c r="P14" s="3" t="n">
         <v>0.1454</v>
       </c>
+      <c r="Q14" s="3" t="n">
+        <v>0.1454</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4332,6 +4545,9 @@
       <c r="P15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4386,6 +4602,9 @@
       <c r="P16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4440,6 +4659,9 @@
       <c r="P17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4494,6 +4716,9 @@
       <c r="P18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4548,6 +4773,9 @@
       <c r="P19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4602,6 +4830,9 @@
       <c r="P20" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q20" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4656,6 +4887,9 @@
       <c r="P21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4710,6 +4944,9 @@
       <c r="P22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4764,6 +5001,9 @@
       <c r="P23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4818,6 +5058,9 @@
       <c r="P24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4872,6 +5115,9 @@
       <c r="P25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4926,6 +5172,9 @@
       <c r="P26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4980,6 +5229,9 @@
       <c r="P27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5034,6 +5286,9 @@
       <c r="P28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5088,6 +5343,9 @@
       <c r="P29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5142,6 +5400,9 @@
       <c r="P30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5196,6 +5457,9 @@
       <c r="P31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5250,6 +5514,9 @@
       <c r="P32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5304,6 +5571,9 @@
       <c r="P33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5358,6 +5628,9 @@
       <c r="P34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5412,6 +5685,9 @@
       <c r="P35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5466,6 +5742,9 @@
       <c r="P36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5520,6 +5799,9 @@
       <c r="P37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5574,6 +5856,9 @@
       <c r="P38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5628,6 +5913,9 @@
       <c r="P39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="Q39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5680,6 +5968,9 @@
         <v>0.13</v>
       </c>
       <c r="P40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="Q40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update treasury bond yields - 2026-05-07
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:R55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -464,6 +464,7 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -552,6 +553,11 @@
           <t>06-May-26</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>06-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -609,6 +615,9 @@
       <c r="Q2" s="3" t="n">
         <v>0.08136666666666668</v>
       </c>
+      <c r="R2" s="3" t="n">
+        <v>0.08145000000000001</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -666,6 +675,9 @@
       <c r="Q3" s="3" t="n">
         <v>0.0818</v>
       </c>
+      <c r="R3" s="3" t="n">
+        <v>0.08180000000000001</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -723,6 +735,9 @@
       <c r="Q4" s="3" t="n">
         <v>0.08318571428571429</v>
       </c>
+      <c r="R4" s="3" t="n">
+        <v>0.08311428571428571</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -780,6 +795,9 @@
       <c r="Q5" s="3" t="n">
         <v>0.08448750000000001</v>
       </c>
+      <c r="R5" s="3" t="n">
+        <v>0.084175</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -837,6 +855,9 @@
       <c r="Q6" s="3" t="n">
         <v>0.08427999999999999</v>
       </c>
+      <c r="R6" s="3" t="n">
+        <v>0.08427999999999999</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -894,6 +915,9 @@
       <c r="Q7" s="3" t="n">
         <v>0.08650000000000001</v>
       </c>
+      <c r="R7" s="3" t="n">
+        <v>0.08657142857142859</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -951,6 +975,9 @@
       <c r="Q8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="R8" s="3" t="n">
+        <v>0.08629999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1008,6 +1035,9 @@
       <c r="Q9" s="3" t="n">
         <v>0.08851999999999999</v>
       </c>
+      <c r="R9" s="3" t="n">
+        <v>0.08851999999999999</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1065,6 +1095,9 @@
       <c r="Q10" s="3" t="n">
         <v>0.0901375</v>
       </c>
+      <c r="R10" s="3" t="n">
+        <v>0.08972857142857142</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1122,6 +1155,9 @@
       <c r="Q11" s="3" t="n">
         <v>0.08984</v>
       </c>
+      <c r="R11" s="3" t="n">
+        <v>0.08984</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1179,6 +1215,9 @@
       <c r="Q12" s="3" t="n">
         <v>0.09111666666666667</v>
       </c>
+      <c r="R12" s="3" t="n">
+        <v>0.09111666666666667</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1236,6 +1275,9 @@
       <c r="Q13" s="3" t="n">
         <v>0.09304999999999998</v>
       </c>
+      <c r="R13" s="3" t="n">
+        <v>0.09329999999999999</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1293,6 +1335,9 @@
       <c r="Q14" s="3" t="n">
         <v>0.09497777777777777</v>
       </c>
+      <c r="R14" s="3" t="n">
+        <v>0.09492222222222221</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1350,6 +1395,9 @@
       <c r="Q15" s="3" t="n">
         <v>0.09484285714285713</v>
       </c>
+      <c r="R15" s="3" t="n">
+        <v>0.09469999999999999</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1407,6 +1455,9 @@
       <c r="Q16" s="3" t="n">
         <v>0.096</v>
       </c>
+      <c r="R16" s="3" t="n">
+        <v>0.09575</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1464,6 +1515,9 @@
       <c r="Q17" s="3" t="n">
         <v>0.09646250000000001</v>
       </c>
+      <c r="R17" s="3" t="n">
+        <v>0.09608750000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1521,6 +1575,9 @@
       <c r="Q18" s="3" t="n">
         <v>0.09648571428571427</v>
       </c>
+      <c r="R18" s="3" t="n">
+        <v>0.0964142857142857</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1578,6 +1635,9 @@
       <c r="Q19" s="3" t="n">
         <v>0.09701249999999999</v>
       </c>
+      <c r="R19" s="3" t="n">
+        <v>0.0968875</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1635,6 +1695,9 @@
       <c r="Q20" s="3" t="n">
         <v>0.09758888888888889</v>
       </c>
+      <c r="R20" s="3" t="n">
+        <v>0.09747777777777777</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1692,6 +1755,9 @@
       <c r="Q21" s="3" t="n">
         <v>0.0968</v>
       </c>
+      <c r="R21" s="3" t="n">
+        <v>0.0968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1749,6 +1815,9 @@
       <c r="Q22" s="3" t="n">
         <v>0.09778333333333333</v>
       </c>
+      <c r="R22" s="3" t="n">
+        <v>0.09770000000000001</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1806,6 +1875,9 @@
       <c r="Q23" s="3" t="n">
         <v>0.09895555555555556</v>
       </c>
+      <c r="R23" s="3" t="n">
+        <v>0.09886666666666669</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1863,6 +1935,9 @@
       <c r="Q24" s="3" t="n">
         <v>0.09758</v>
       </c>
+      <c r="R24" s="3" t="n">
+        <v>0.09758</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1920,6 +1995,9 @@
       <c r="Q25" s="3" t="n">
         <v>0.09928750000000001</v>
       </c>
+      <c r="R25" s="3" t="n">
+        <v>0.0991625</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1977,6 +2055,9 @@
       <c r="Q26" s="3" t="n">
         <v>0.09958750000000001</v>
       </c>
+      <c r="R26" s="3" t="n">
+        <v>0.0994625</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2034,6 +2115,9 @@
       <c r="Q27" s="3" t="n">
         <v>0.1000666666666667</v>
       </c>
+      <c r="R27" s="3" t="n">
+        <v>0.1000111111111111</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2091,6 +2175,9 @@
       <c r="Q28" s="3" t="n">
         <v>0.100375</v>
       </c>
+      <c r="R28" s="3" t="n">
+        <v>0.10035</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2148,6 +2235,9 @@
       <c r="Q29" s="3" t="n">
         <v>0.10025</v>
       </c>
+      <c r="R29" s="3" t="n">
+        <v>0.1001666666666667</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2205,6 +2295,9 @@
       <c r="Q30" s="3" t="n">
         <v>0.1008</v>
       </c>
+      <c r="R30" s="3" t="n">
+        <v>0.1007285714285714</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2262,6 +2355,9 @@
       <c r="Q31" s="3" t="n">
         <v>0.1008666666666667</v>
       </c>
+      <c r="R31" s="3" t="n">
+        <v>0.1008666666666667</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2319,6 +2415,9 @@
       <c r="Q32" s="3" t="n">
         <v>0.10185</v>
       </c>
+      <c r="R32" s="3" t="n">
+        <v>0.1017125</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2376,6 +2475,9 @@
       <c r="Q33" s="3" t="n">
         <v>0.1018333333333333</v>
       </c>
+      <c r="R33" s="3" t="n">
+        <v>0.1019166666666667</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2433,6 +2535,9 @@
       <c r="Q34" s="3" t="n">
         <v>0.102</v>
       </c>
+      <c r="R34" s="3" t="n">
+        <v>0.102</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2490,6 +2595,9 @@
       <c r="Q35" s="3" t="n">
         <v>0.1043</v>
       </c>
+      <c r="R35" s="3" t="n">
+        <v>0.1043</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2547,6 +2655,9 @@
       <c r="Q36" s="3" t="n">
         <v>0.1058333333333333</v>
       </c>
+      <c r="R36" s="3" t="n">
+        <v>0.1058333333333333</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2604,6 +2715,9 @@
       <c r="Q37" s="3" t="n">
         <v>0.10685</v>
       </c>
+      <c r="R37" s="3" t="n">
+        <v>0.1067875</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2661,6 +2775,9 @@
       <c r="Q38" s="3" t="n">
         <v>0.10781</v>
       </c>
+      <c r="R38" s="3" t="n">
+        <v>0.1076222222222222</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2718,6 +2835,9 @@
       <c r="Q39" s="3" t="n">
         <v>0.10828</v>
       </c>
+      <c r="R39" s="3" t="n">
+        <v>0.10828</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2775,6 +2895,9 @@
       <c r="Q40" s="3" t="n">
         <v>0.1098555555555555</v>
       </c>
+      <c r="R40" s="3" t="n">
+        <v>0.1098555555555555</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2832,6 +2955,9 @@
       <c r="Q41" s="3" t="n">
         <v>0.10896</v>
       </c>
+      <c r="R41" s="3" t="n">
+        <v>0.10896</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2889,6 +3015,9 @@
       <c r="Q42" s="3" t="n">
         <v>0.1099375</v>
       </c>
+      <c r="R42" s="3" t="n">
+        <v>0.1099375</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2946,6 +3075,9 @@
       <c r="Q43" s="3" t="n">
         <v>0.10952</v>
       </c>
+      <c r="R43" s="3" t="n">
+        <v>0.10952</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3003,6 +3135,9 @@
       <c r="Q44" s="3" t="n">
         <v>0.110975</v>
       </c>
+      <c r="R44" s="3" t="n">
+        <v>0.1111625</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3060,6 +3195,9 @@
       <c r="Q45" s="3" t="n">
         <v>0.1105333333333333</v>
       </c>
+      <c r="R45" s="3" t="n">
+        <v>0.1106166666666667</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3117,6 +3255,9 @@
       <c r="Q46" s="3" t="n">
         <v>0.1101</v>
       </c>
+      <c r="R46" s="3" t="n">
+        <v>0.1101</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3174,6 +3315,9 @@
       <c r="Q47" s="3" t="n">
         <v>0.111325</v>
       </c>
+      <c r="R47" s="3" t="n">
+        <v>0.11155</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3231,6 +3375,9 @@
       <c r="Q48" s="3" t="n">
         <v>0.1112166666666667</v>
       </c>
+      <c r="R48" s="3" t="n">
+        <v>0.1112166666666667</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3288,6 +3435,9 @@
       <c r="Q49" s="3" t="n">
         <v>0.1118571428571429</v>
       </c>
+      <c r="R49" s="3" t="n">
+        <v>0.1119285714285714</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3345,6 +3495,9 @@
       <c r="Q50" s="3" t="n">
         <v>0.1116</v>
       </c>
+      <c r="R50" s="3" t="n">
+        <v>0.1116</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3402,6 +3555,9 @@
       <c r="Q51" s="3" t="n">
         <v>0.112625</v>
       </c>
+      <c r="R51" s="3" t="n">
+        <v>0.112625</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3459,6 +3615,9 @@
       <c r="Q52" s="3" t="n">
         <v>0.1135</v>
       </c>
+      <c r="R52" s="3" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3516,6 +3675,9 @@
       <c r="Q53" s="3" t="n">
         <v>0.114</v>
       </c>
+      <c r="R53" s="3" t="n">
+        <v>0.114</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3573,6 +3735,9 @@
       <c r="Q54" s="3" t="n">
         <v>0.1145</v>
       </c>
+      <c r="R54" s="3" t="n">
+        <v>0.1145</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3628,6 +3793,9 @@
         <v>0.1165</v>
       </c>
       <c r="Q55" s="3" t="n">
+        <v>0.1165</v>
+      </c>
+      <c r="R55" s="3" t="n">
         <v>0.1165</v>
       </c>
     </row>
@@ -3642,7 +3810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:R40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3662,6 +3830,7 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3750,6 +3919,11 @@
           <t>06-May-26</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>06-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3807,6 +3981,9 @@
       <c r="Q2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3864,6 +4041,9 @@
       <c r="Q3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="R3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3921,6 +4101,9 @@
       <c r="Q4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3978,6 +4161,9 @@
       <c r="Q5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="R5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4035,6 +4221,9 @@
       <c r="Q6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4092,6 +4281,9 @@
       <c r="Q7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4149,6 +4341,9 @@
       <c r="Q8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4206,6 +4401,9 @@
       <c r="Q9" s="3" t="n">
         <v>0.1444</v>
       </c>
+      <c r="R9" s="3" t="n">
+        <v>0.1444</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4263,6 +4461,9 @@
       <c r="Q10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4320,6 +4521,9 @@
       <c r="Q11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4377,6 +4581,9 @@
       <c r="Q12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4434,6 +4641,9 @@
       <c r="Q13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4491,6 +4701,9 @@
       <c r="Q14" s="3" t="n">
         <v>0.1454</v>
       </c>
+      <c r="R14" s="3" t="n">
+        <v>0.1454</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4548,6 +4761,9 @@
       <c r="Q15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4605,6 +4821,9 @@
       <c r="Q16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4662,6 +4881,9 @@
       <c r="Q17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4719,6 +4941,9 @@
       <c r="Q18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4776,6 +5001,9 @@
       <c r="Q19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4833,6 +5061,9 @@
       <c r="Q20" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R20" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4890,6 +5121,9 @@
       <c r="Q21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4947,6 +5181,9 @@
       <c r="Q22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5004,6 +5241,9 @@
       <c r="Q23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5061,6 +5301,9 @@
       <c r="Q24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -5118,6 +5361,9 @@
       <c r="Q25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -5175,6 +5421,9 @@
       <c r="Q26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5232,6 +5481,9 @@
       <c r="Q27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5289,6 +5541,9 @@
       <c r="Q28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5346,6 +5601,9 @@
       <c r="Q29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5403,6 +5661,9 @@
       <c r="Q30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5460,6 +5721,9 @@
       <c r="Q31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5517,6 +5781,9 @@
       <c r="Q32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5574,6 +5841,9 @@
       <c r="Q33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5631,6 +5901,9 @@
       <c r="Q34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5688,6 +5961,9 @@
       <c r="Q35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5745,6 +6021,9 @@
       <c r="Q36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5802,6 +6081,9 @@
       <c r="Q37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5859,6 +6141,9 @@
       <c r="Q38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5916,6 +6201,9 @@
       <c r="Q39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="R39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5971,6 +6259,9 @@
         <v>0.13</v>
       </c>
       <c r="Q40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="R40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update treasury bond yields - 2026-05-08
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:S55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -465,6 +465,7 @@
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -558,6 +559,11 @@
           <t>06-May-26</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>07-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -618,6 +624,9 @@
       <c r="R2" s="3" t="n">
         <v>0.08145000000000001</v>
       </c>
+      <c r="S2" s="3" t="n">
+        <v>0.08070000000000001</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -678,6 +687,9 @@
       <c r="R3" s="3" t="n">
         <v>0.08180000000000001</v>
       </c>
+      <c r="S3" s="3" t="n">
+        <v>0.08163333333333335</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -738,6 +750,9 @@
       <c r="R4" s="3" t="n">
         <v>0.08311428571428571</v>
       </c>
+      <c r="S4" s="3" t="n">
+        <v>0.08297142857142857</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -798,6 +813,9 @@
       <c r="R5" s="3" t="n">
         <v>0.084175</v>
       </c>
+      <c r="S5" s="3" t="n">
+        <v>0.08426666666666666</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -858,6 +876,9 @@
       <c r="R6" s="3" t="n">
         <v>0.08427999999999999</v>
       </c>
+      <c r="S6" s="3" t="n">
+        <v>0.08427999999999999</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -918,6 +939,9 @@
       <c r="R7" s="3" t="n">
         <v>0.08657142857142859</v>
       </c>
+      <c r="S7" s="3" t="n">
+        <v>0.08642857142857144</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -978,6 +1002,9 @@
       <c r="R8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="S8" s="3" t="n">
+        <v>0.08629999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1038,6 +1065,9 @@
       <c r="R9" s="3" t="n">
         <v>0.08851999999999999</v>
       </c>
+      <c r="S9" s="3" t="n">
+        <v>0.08851999999999999</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1098,6 +1128,9 @@
       <c r="R10" s="3" t="n">
         <v>0.08972857142857142</v>
       </c>
+      <c r="S10" s="3" t="n">
+        <v>0.08972857142857142</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1158,6 +1191,9 @@
       <c r="R11" s="3" t="n">
         <v>0.08984</v>
       </c>
+      <c r="S11" s="3" t="n">
+        <v>0.08984</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1218,6 +1254,9 @@
       <c r="R12" s="3" t="n">
         <v>0.09111666666666667</v>
       </c>
+      <c r="S12" s="3" t="n">
+        <v>0.09111666666666667</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1278,6 +1317,9 @@
       <c r="R13" s="3" t="n">
         <v>0.09329999999999999</v>
       </c>
+      <c r="S13" s="3" t="n">
+        <v>0.09313333333333333</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1338,6 +1380,9 @@
       <c r="R14" s="3" t="n">
         <v>0.09492222222222221</v>
       </c>
+      <c r="S14" s="3" t="n">
+        <v>0.09470000000000001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1398,6 +1443,9 @@
       <c r="R15" s="3" t="n">
         <v>0.09469999999999999</v>
       </c>
+      <c r="S15" s="3" t="n">
+        <v>0.09448571428571428</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1458,6 +1506,9 @@
       <c r="R16" s="3" t="n">
         <v>0.09575</v>
       </c>
+      <c r="S16" s="3" t="n">
+        <v>0.09568750000000001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1518,6 +1569,9 @@
       <c r="R17" s="3" t="n">
         <v>0.09608750000000001</v>
       </c>
+      <c r="S17" s="3" t="n">
+        <v>0.09589999999999999</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1578,6 +1632,9 @@
       <c r="R18" s="3" t="n">
         <v>0.0964142857142857</v>
       </c>
+      <c r="S18" s="3" t="n">
+        <v>0.09619999999999998</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1638,6 +1695,9 @@
       <c r="R19" s="3" t="n">
         <v>0.0968875</v>
       </c>
+      <c r="S19" s="3" t="n">
+        <v>0.09661249999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1698,6 +1758,9 @@
       <c r="R20" s="3" t="n">
         <v>0.09747777777777777</v>
       </c>
+      <c r="S20" s="3" t="n">
+        <v>0.09725555555555555</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1758,6 +1821,9 @@
       <c r="R21" s="3" t="n">
         <v>0.0968</v>
       </c>
+      <c r="S21" s="3" t="n">
+        <v>0.0968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1818,6 +1884,9 @@
       <c r="R22" s="3" t="n">
         <v>0.09770000000000001</v>
       </c>
+      <c r="S22" s="3" t="n">
+        <v>0.09770000000000001</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1878,6 +1947,9 @@
       <c r="R23" s="3" t="n">
         <v>0.09886666666666669</v>
       </c>
+      <c r="S23" s="3" t="n">
+        <v>0.09808888888888889</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1938,6 +2010,9 @@
       <c r="R24" s="3" t="n">
         <v>0.09758</v>
       </c>
+      <c r="S24" s="3" t="n">
+        <v>0.09758</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1998,6 +2073,9 @@
       <c r="R25" s="3" t="n">
         <v>0.0991625</v>
       </c>
+      <c r="S25" s="3" t="n">
+        <v>0.09857500000000001</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2058,6 +2136,9 @@
       <c r="R26" s="3" t="n">
         <v>0.0994625</v>
       </c>
+      <c r="S26" s="3" t="n">
+        <v>0.0989</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2118,6 +2199,9 @@
       <c r="R27" s="3" t="n">
         <v>0.1000111111111111</v>
       </c>
+      <c r="S27" s="3" t="n">
+        <v>0.09945555555555556</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2178,6 +2262,9 @@
       <c r="R28" s="3" t="n">
         <v>0.10035</v>
       </c>
+      <c r="S28" s="3" t="n">
+        <v>0.0999625</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2238,6 +2325,9 @@
       <c r="R29" s="3" t="n">
         <v>0.1001666666666667</v>
       </c>
+      <c r="S29" s="3" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2298,6 +2388,9 @@
       <c r="R30" s="3" t="n">
         <v>0.1007285714285714</v>
       </c>
+      <c r="S30" s="3" t="n">
+        <v>0.1004714285714286</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2358,6 +2451,9 @@
       <c r="R31" s="3" t="n">
         <v>0.1008666666666667</v>
       </c>
+      <c r="S31" s="3" t="n">
+        <v>0.1007833333333333</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2418,6 +2514,9 @@
       <c r="R32" s="3" t="n">
         <v>0.1017125</v>
       </c>
+      <c r="S32" s="3" t="n">
+        <v>0.1014285714285714</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2478,6 +2577,9 @@
       <c r="R33" s="3" t="n">
         <v>0.1019166666666667</v>
       </c>
+      <c r="S33" s="3" t="n">
+        <v>0.1019166666666667</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2538,6 +2640,9 @@
       <c r="R34" s="3" t="n">
         <v>0.102</v>
       </c>
+      <c r="S34" s="3" t="n">
+        <v>0.102</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2598,6 +2703,9 @@
       <c r="R35" s="3" t="n">
         <v>0.1043</v>
       </c>
+      <c r="S35" s="3" t="n">
+        <v>0.1043</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2658,6 +2766,9 @@
       <c r="R36" s="3" t="n">
         <v>0.1058333333333333</v>
       </c>
+      <c r="S36" s="3" t="n">
+        <v>0.1058333333333333</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2718,6 +2829,9 @@
       <c r="R37" s="3" t="n">
         <v>0.1067875</v>
       </c>
+      <c r="S37" s="3" t="n">
+        <v>0.1064125</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2778,6 +2892,9 @@
       <c r="R38" s="3" t="n">
         <v>0.1076222222222222</v>
       </c>
+      <c r="S38" s="3" t="n">
+        <v>0.1072333333333333</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2838,6 +2955,9 @@
       <c r="R39" s="3" t="n">
         <v>0.10828</v>
       </c>
+      <c r="S39" s="3" t="n">
+        <v>0.10808</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2898,6 +3018,9 @@
       <c r="R40" s="3" t="n">
         <v>0.1098555555555555</v>
       </c>
+      <c r="S40" s="3" t="n">
+        <v>0.1094111111111111</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2958,6 +3081,9 @@
       <c r="R41" s="3" t="n">
         <v>0.10896</v>
       </c>
+      <c r="S41" s="3" t="n">
+        <v>0.10876</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3018,6 +3144,9 @@
       <c r="R42" s="3" t="n">
         <v>0.1099375</v>
       </c>
+      <c r="S42" s="3" t="n">
+        <v>0.1094375</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3078,6 +3207,9 @@
       <c r="R43" s="3" t="n">
         <v>0.10952</v>
       </c>
+      <c r="S43" s="3" t="n">
+        <v>0.10952</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3138,6 +3270,9 @@
       <c r="R44" s="3" t="n">
         <v>0.1111625</v>
       </c>
+      <c r="S44" s="3" t="n">
+        <v>0.1106875</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3198,6 +3333,9 @@
       <c r="R45" s="3" t="n">
         <v>0.1106166666666667</v>
       </c>
+      <c r="S45" s="3" t="n">
+        <v>0.1103666666666667</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3258,6 +3396,9 @@
       <c r="R46" s="3" t="n">
         <v>0.1101</v>
       </c>
+      <c r="S46" s="3" t="n">
+        <v>0.1101</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3318,6 +3459,9 @@
       <c r="R47" s="3" t="n">
         <v>0.11155</v>
       </c>
+      <c r="S47" s="3" t="n">
+        <v>0.1109857142857143</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3378,6 +3522,9 @@
       <c r="R48" s="3" t="n">
         <v>0.1112166666666667</v>
       </c>
+      <c r="S48" s="3" t="n">
+        <v>0.11105</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3438,6 +3585,9 @@
       <c r="R49" s="3" t="n">
         <v>0.1119285714285714</v>
       </c>
+      <c r="S49" s="3" t="n">
+        <v>0.1119285714285714</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3498,6 +3648,9 @@
       <c r="R50" s="3" t="n">
         <v>0.1116</v>
       </c>
+      <c r="S50" s="3" t="n">
+        <v>0.1116</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3558,6 +3711,9 @@
       <c r="R51" s="3" t="n">
         <v>0.112625</v>
       </c>
+      <c r="S51" s="3" t="n">
+        <v>0.112625</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3618,6 +3774,9 @@
       <c r="R52" s="3" t="n">
         <v>0.1135</v>
       </c>
+      <c r="S52" s="3" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3678,6 +3837,9 @@
       <c r="R53" s="3" t="n">
         <v>0.114</v>
       </c>
+      <c r="S53" s="3" t="n">
+        <v>0.114</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3738,6 +3900,9 @@
       <c r="R54" s="3" t="n">
         <v>0.1145</v>
       </c>
+      <c r="S54" s="3" t="n">
+        <v>0.1145</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3796,6 +3961,9 @@
         <v>0.1165</v>
       </c>
       <c r="R55" s="3" t="n">
+        <v>0.1165</v>
+      </c>
+      <c r="S55" s="3" t="n">
         <v>0.1165</v>
       </c>
     </row>
@@ -3810,7 +3978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3831,6 +3999,7 @@
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3924,6 +4093,11 @@
           <t>06-May-26</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>07-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3984,6 +4158,9 @@
       <c r="R2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4044,6 +4221,9 @@
       <c r="R3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="S3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4104,6 +4284,9 @@
       <c r="R4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4164,6 +4347,9 @@
       <c r="R5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="S5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4224,6 +4410,9 @@
       <c r="R6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4284,6 +4473,9 @@
       <c r="R7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4344,6 +4536,9 @@
       <c r="R8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4404,6 +4599,9 @@
       <c r="R9" s="3" t="n">
         <v>0.1444</v>
       </c>
+      <c r="S9" s="3" t="n">
+        <v>0.1444</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4464,6 +4662,9 @@
       <c r="R10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4524,6 +4725,9 @@
       <c r="R11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4584,6 +4788,9 @@
       <c r="R12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4644,6 +4851,9 @@
       <c r="R13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4704,6 +4914,9 @@
       <c r="R14" s="3" t="n">
         <v>0.1454</v>
       </c>
+      <c r="S14" s="3" t="n">
+        <v>0.1454</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4764,6 +4977,9 @@
       <c r="R15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4824,6 +5040,9 @@
       <c r="R16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4884,6 +5103,9 @@
       <c r="R17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4944,6 +5166,9 @@
       <c r="R18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5004,6 +5229,9 @@
       <c r="R19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5064,6 +5292,9 @@
       <c r="R20" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S20" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5124,6 +5355,9 @@
       <c r="R21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5184,6 +5418,9 @@
       <c r="R22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5244,6 +5481,9 @@
       <c r="R23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5304,6 +5544,9 @@
       <c r="R24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -5364,6 +5607,9 @@
       <c r="R25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -5424,6 +5670,9 @@
       <c r="R26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5484,6 +5733,9 @@
       <c r="R27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5544,6 +5796,9 @@
       <c r="R28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5604,6 +5859,9 @@
       <c r="R29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5664,6 +5922,9 @@
       <c r="R30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5724,6 +5985,9 @@
       <c r="R31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5784,6 +6048,9 @@
       <c r="R32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5844,6 +6111,9 @@
       <c r="R33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5904,6 +6174,9 @@
       <c r="R34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5964,6 +6237,9 @@
       <c r="R35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6024,6 +6300,9 @@
       <c r="R36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6084,6 +6363,9 @@
       <c r="R37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6144,6 +6426,9 @@
       <c r="R38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6204,6 +6489,9 @@
       <c r="R39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="S39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6262,6 +6550,9 @@
         <v>0.13</v>
       </c>
       <c r="R40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="S40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update treasury bond yields - 2026-05-12
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S55"/>
+  <dimension ref="A1:T55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -466,6 +466,7 @@
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,6 +565,11 @@
           <t>07-May-26</t>
         </is>
       </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -627,6 +633,9 @@
       <c r="S2" s="3" t="n">
         <v>0.08070000000000001</v>
       </c>
+      <c r="T2" s="3" t="n">
+        <v>0.08120000000000001</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -690,6 +699,9 @@
       <c r="S3" s="3" t="n">
         <v>0.08163333333333335</v>
       </c>
+      <c r="T3" s="3" t="n">
+        <v>0.08155000000000001</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -753,6 +765,9 @@
       <c r="S4" s="3" t="n">
         <v>0.08297142857142857</v>
       </c>
+      <c r="T4" s="3" t="n">
+        <v>0.0830375</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -816,6 +831,9 @@
       <c r="S5" s="3" t="n">
         <v>0.08426666666666666</v>
       </c>
+      <c r="T5" s="3" t="n">
+        <v>0.08415555555555555</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -879,6 +897,9 @@
       <c r="S6" s="3" t="n">
         <v>0.08427999999999999</v>
       </c>
+      <c r="T6" s="3" t="n">
+        <v>0.08427999999999999</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -942,6 +963,9 @@
       <c r="S7" s="3" t="n">
         <v>0.08642857142857144</v>
       </c>
+      <c r="T7" s="3" t="n">
+        <v>0.0862857142857143</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1005,6 +1029,9 @@
       <c r="S8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="T8" s="3" t="n">
+        <v>0.08629999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1068,6 +1095,9 @@
       <c r="S9" s="3" t="n">
         <v>0.08851999999999999</v>
       </c>
+      <c r="T9" s="3" t="n">
+        <v>0.08851999999999999</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1131,6 +1161,9 @@
       <c r="S10" s="3" t="n">
         <v>0.08972857142857142</v>
       </c>
+      <c r="T10" s="3" t="n">
+        <v>0.08972857142857142</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1194,6 +1227,9 @@
       <c r="S11" s="3" t="n">
         <v>0.08984</v>
       </c>
+      <c r="T11" s="3" t="n">
+        <v>0.08984</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1257,6 +1293,9 @@
       <c r="S12" s="3" t="n">
         <v>0.09111666666666667</v>
       </c>
+      <c r="T12" s="3" t="n">
+        <v>0.09111666666666667</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1320,6 +1359,9 @@
       <c r="S13" s="3" t="n">
         <v>0.09313333333333333</v>
       </c>
+      <c r="T13" s="3" t="n">
+        <v>0.09304999999999998</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1383,6 +1425,9 @@
       <c r="S14" s="3" t="n">
         <v>0.09470000000000001</v>
       </c>
+      <c r="T14" s="3" t="n">
+        <v>0.09497777777777777</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1446,6 +1491,9 @@
       <c r="S15" s="3" t="n">
         <v>0.09448571428571428</v>
       </c>
+      <c r="T15" s="3" t="n">
+        <v>0.09469999999999999</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1509,6 +1557,9 @@
       <c r="S16" s="3" t="n">
         <v>0.09568750000000001</v>
       </c>
+      <c r="T16" s="3" t="n">
+        <v>0.09581249999999999</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1572,6 +1623,9 @@
       <c r="S17" s="3" t="n">
         <v>0.09589999999999999</v>
       </c>
+      <c r="T17" s="3" t="n">
+        <v>0.096025</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1635,6 +1689,9 @@
       <c r="S18" s="3" t="n">
         <v>0.09619999999999998</v>
       </c>
+      <c r="T18" s="3" t="n">
+        <v>0.09619999999999999</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1698,6 +1755,9 @@
       <c r="S19" s="3" t="n">
         <v>0.09661249999999999</v>
       </c>
+      <c r="T19" s="3" t="n">
+        <v>0.09663749999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1761,6 +1821,9 @@
       <c r="S20" s="3" t="n">
         <v>0.09725555555555555</v>
       </c>
+      <c r="T20" s="3" t="n">
+        <v>0.09714444444444444</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1824,6 +1887,9 @@
       <c r="S21" s="3" t="n">
         <v>0.0968</v>
       </c>
+      <c r="T21" s="3" t="n">
+        <v>0.0968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1887,6 +1953,9 @@
       <c r="S22" s="3" t="n">
         <v>0.09770000000000001</v>
       </c>
+      <c r="T22" s="3" t="n">
+        <v>0.09714</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1950,6 +2019,9 @@
       <c r="S23" s="3" t="n">
         <v>0.09808888888888889</v>
       </c>
+      <c r="T23" s="3" t="n">
+        <v>0.09803333333333335</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2013,6 +2085,9 @@
       <c r="S24" s="3" t="n">
         <v>0.09758</v>
       </c>
+      <c r="T24" s="3" t="n">
+        <v>0.09758</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2076,6 +2151,9 @@
       <c r="S25" s="3" t="n">
         <v>0.09857500000000001</v>
       </c>
+      <c r="T25" s="3" t="n">
+        <v>0.0985375</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2139,6 +2217,9 @@
       <c r="S26" s="3" t="n">
         <v>0.0989</v>
       </c>
+      <c r="T26" s="3" t="n">
+        <v>0.098775</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2202,6 +2283,9 @@
       <c r="S27" s="3" t="n">
         <v>0.09945555555555556</v>
       </c>
+      <c r="T27" s="3" t="n">
+        <v>0.09951111111111111</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2265,6 +2349,9 @@
       <c r="S28" s="3" t="n">
         <v>0.0999625</v>
       </c>
+      <c r="T28" s="3" t="n">
+        <v>0.1000625</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2328,6 +2415,9 @@
       <c r="S29" s="3" t="n">
         <v>0.1</v>
       </c>
+      <c r="T29" s="3" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2391,6 +2481,9 @@
       <c r="S30" s="3" t="n">
         <v>0.1004714285714286</v>
       </c>
+      <c r="T30" s="3" t="n">
+        <v>0.1004428571428572</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2454,6 +2547,9 @@
       <c r="S31" s="3" t="n">
         <v>0.1007833333333333</v>
       </c>
+      <c r="T31" s="3" t="n">
+        <v>0.1006166666666666</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2517,6 +2613,9 @@
       <c r="S32" s="3" t="n">
         <v>0.1014285714285714</v>
       </c>
+      <c r="T32" s="3" t="n">
+        <v>0.1014285714285714</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2580,6 +2679,9 @@
       <c r="S33" s="3" t="n">
         <v>0.1019166666666667</v>
       </c>
+      <c r="T33" s="3" t="n">
+        <v>0.10175</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2643,6 +2745,9 @@
       <c r="S34" s="3" t="n">
         <v>0.102</v>
       </c>
+      <c r="T34" s="3" t="n">
+        <v>0.102</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2706,6 +2811,9 @@
       <c r="S35" s="3" t="n">
         <v>0.1043</v>
       </c>
+      <c r="T35" s="3" t="n">
+        <v>0.1043</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2769,6 +2877,9 @@
       <c r="S36" s="3" t="n">
         <v>0.1058333333333333</v>
       </c>
+      <c r="T36" s="3" t="n">
+        <v>0.1058333333333333</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2832,6 +2943,9 @@
       <c r="S37" s="3" t="n">
         <v>0.1064125</v>
       </c>
+      <c r="T37" s="3" t="n">
+        <v>0.1066</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2895,6 +3009,9 @@
       <c r="S38" s="3" t="n">
         <v>0.1072333333333333</v>
       </c>
+      <c r="T38" s="3" t="n">
+        <v>0.10746</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2958,6 +3075,9 @@
       <c r="S39" s="3" t="n">
         <v>0.10808</v>
       </c>
+      <c r="T39" s="3" t="n">
+        <v>0.10808</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3021,6 +3141,9 @@
       <c r="S40" s="3" t="n">
         <v>0.1094111111111111</v>
       </c>
+      <c r="T40" s="3" t="n">
+        <v>0.1092444444444444</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3084,6 +3207,9 @@
       <c r="S41" s="3" t="n">
         <v>0.10876</v>
       </c>
+      <c r="T41" s="3" t="n">
+        <v>0.10876</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3147,6 +3273,9 @@
       <c r="S42" s="3" t="n">
         <v>0.1094375</v>
       </c>
+      <c r="T42" s="3" t="n">
+        <v>0.1095</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3210,6 +3339,9 @@
       <c r="S43" s="3" t="n">
         <v>0.10952</v>
       </c>
+      <c r="T43" s="3" t="n">
+        <v>0.10942</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3273,6 +3405,9 @@
       <c r="S44" s="3" t="n">
         <v>0.1106875</v>
       </c>
+      <c r="T44" s="3" t="n">
+        <v>0.1106375</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3336,6 +3471,9 @@
       <c r="S45" s="3" t="n">
         <v>0.1103666666666667</v>
       </c>
+      <c r="T45" s="3" t="n">
+        <v>0.1102333333333333</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3399,6 +3537,9 @@
       <c r="S46" s="3" t="n">
         <v>0.1101</v>
       </c>
+      <c r="T46" s="3" t="n">
+        <v>0.1108</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3462,6 +3603,9 @@
       <c r="S47" s="3" t="n">
         <v>0.1109857142857143</v>
       </c>
+      <c r="T47" s="3" t="n">
+        <v>0.1114142857142857</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3525,6 +3669,9 @@
       <c r="S48" s="3" t="n">
         <v>0.11105</v>
       </c>
+      <c r="T48" s="3" t="n">
+        <v>0.111</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3588,6 +3735,9 @@
       <c r="S49" s="3" t="n">
         <v>0.1119285714285714</v>
       </c>
+      <c r="T49" s="3" t="n">
+        <v>0.1115833333333333</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3651,6 +3801,9 @@
       <c r="S50" s="3" t="n">
         <v>0.1116</v>
       </c>
+      <c r="T50" s="3" t="n">
+        <v>0.1116</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3714,6 +3867,9 @@
       <c r="S51" s="3" t="n">
         <v>0.112625</v>
       </c>
+      <c r="T51" s="3" t="n">
+        <v>0.112625</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3777,6 +3933,9 @@
       <c r="S52" s="3" t="n">
         <v>0.1135</v>
       </c>
+      <c r="T52" s="3" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3840,6 +3999,9 @@
       <c r="S53" s="3" t="n">
         <v>0.114</v>
       </c>
+      <c r="T53" s="3" t="n">
+        <v>0.114</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3903,6 +4065,9 @@
       <c r="S54" s="3" t="n">
         <v>0.1145</v>
       </c>
+      <c r="T54" s="3" t="n">
+        <v>0.1145</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3964,6 +4129,9 @@
         <v>0.1165</v>
       </c>
       <c r="S55" s="3" t="n">
+        <v>0.1165</v>
+      </c>
+      <c r="T55" s="3" t="n">
         <v>0.1165</v>
       </c>
     </row>
@@ -3978,7 +4146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S40"/>
+  <dimension ref="A1:T40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4000,6 +4168,7 @@
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4098,6 +4267,11 @@
           <t>07-May-26</t>
         </is>
       </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4161,6 +4335,9 @@
       <c r="S2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4224,6 +4401,9 @@
       <c r="S3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="T3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4287,6 +4467,9 @@
       <c r="S4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4350,6 +4533,9 @@
       <c r="S5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="T5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4413,6 +4599,9 @@
       <c r="S6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4476,6 +4665,9 @@
       <c r="S7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4539,6 +4731,9 @@
       <c r="S8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4602,6 +4797,9 @@
       <c r="S9" s="3" t="n">
         <v>0.1444</v>
       </c>
+      <c r="T9" s="3" t="n">
+        <v>0.1444</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4665,6 +4863,9 @@
       <c r="S10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4728,6 +4929,9 @@
       <c r="S11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4791,6 +4995,9 @@
       <c r="S12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4854,6 +5061,9 @@
       <c r="S13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4917,6 +5127,9 @@
       <c r="S14" s="3" t="n">
         <v>0.1454</v>
       </c>
+      <c r="T14" s="3" t="n">
+        <v>0.1454</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4980,6 +5193,9 @@
       <c r="S15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5043,6 +5259,9 @@
       <c r="S16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5106,6 +5325,9 @@
       <c r="S17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5169,6 +5391,9 @@
       <c r="S18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5232,6 +5457,9 @@
       <c r="S19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5295,6 +5523,9 @@
       <c r="S20" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T20" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5358,6 +5589,9 @@
       <c r="S21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5421,6 +5655,9 @@
       <c r="S22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5484,6 +5721,9 @@
       <c r="S23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5547,6 +5787,9 @@
       <c r="S24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -5610,6 +5853,9 @@
       <c r="S25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -5673,6 +5919,9 @@
       <c r="S26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5736,6 +5985,9 @@
       <c r="S27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5799,6 +6051,9 @@
       <c r="S28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5862,6 +6117,9 @@
       <c r="S29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5925,6 +6183,9 @@
       <c r="S30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5988,6 +6249,9 @@
       <c r="S31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -6051,6 +6315,9 @@
       <c r="S32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6114,6 +6381,9 @@
       <c r="S33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6177,6 +6447,9 @@
       <c r="S34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6240,6 +6513,9 @@
       <c r="S35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6303,6 +6579,9 @@
       <c r="S36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6366,6 +6645,9 @@
       <c r="S37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6429,6 +6711,9 @@
       <c r="S38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6492,6 +6777,9 @@
       <c r="S39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="T39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6553,6 +6841,9 @@
         <v>0.13</v>
       </c>
       <c r="S40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="T40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update treasury bond yields - 2026-05-13
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -70,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -79,6 +79,7 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T55"/>
+  <dimension ref="A1:U56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -467,6 +468,7 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -570,6 +572,11 @@
           <t>11-May-26</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>12-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -636,6 +643,9 @@
       <c r="T2" s="3" t="n">
         <v>0.08120000000000001</v>
       </c>
+      <c r="U2" s="3" t="n">
+        <v>0.08028333333333335</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -702,6 +712,9 @@
       <c r="T3" s="3" t="n">
         <v>0.08155000000000001</v>
       </c>
+      <c r="U3" s="3" t="n">
+        <v>0.08130000000000001</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -768,6 +781,9 @@
       <c r="T4" s="3" t="n">
         <v>0.0830375</v>
       </c>
+      <c r="U4" s="3" t="n">
+        <v>0.08259999999999999</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -834,6 +850,9 @@
       <c r="T5" s="3" t="n">
         <v>0.08415555555555555</v>
       </c>
+      <c r="U5" s="3" t="n">
+        <v>0.08415555555555555</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -900,6 +919,9 @@
       <c r="T6" s="3" t="n">
         <v>0.08427999999999999</v>
       </c>
+      <c r="U6" s="3" t="n">
+        <v>0.08448</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -966,6 +988,9 @@
       <c r="T7" s="3" t="n">
         <v>0.0862857142857143</v>
       </c>
+      <c r="U7" s="3" t="n">
+        <v>0.08642857142857142</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1032,6 +1057,9 @@
       <c r="T8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="U8" s="3" t="n">
+        <v>0.08629999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1098,6 +1126,9 @@
       <c r="T9" s="3" t="n">
         <v>0.08851999999999999</v>
       </c>
+      <c r="U9" s="3" t="n">
+        <v>0.08882</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1164,6 +1195,9 @@
       <c r="T10" s="3" t="n">
         <v>0.08972857142857142</v>
       </c>
+      <c r="U10" s="3" t="n">
+        <v>0.0898</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1230,6 +1264,9 @@
       <c r="T11" s="3" t="n">
         <v>0.08984</v>
       </c>
+      <c r="U11" s="3" t="n">
+        <v>0.09014</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1296,6 +1333,9 @@
       <c r="T12" s="3" t="n">
         <v>0.09111666666666667</v>
       </c>
+      <c r="U12" s="3" t="n">
+        <v>0.09144999999999999</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1362,6 +1402,9 @@
       <c r="T13" s="3" t="n">
         <v>0.09304999999999998</v>
       </c>
+      <c r="U13" s="3" t="n">
+        <v>0.09346666666666666</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1428,6 +1471,9 @@
       <c r="T14" s="3" t="n">
         <v>0.09497777777777777</v>
       </c>
+      <c r="U14" s="3" t="n">
+        <v>0.09514444444444443</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1494,6 +1540,9 @@
       <c r="T15" s="3" t="n">
         <v>0.09469999999999999</v>
       </c>
+      <c r="U15" s="3" t="n">
+        <v>0.0949857142857143</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1560,6 +1609,9 @@
       <c r="T16" s="3" t="n">
         <v>0.09581249999999999</v>
       </c>
+      <c r="U16" s="3" t="n">
+        <v>0.09612500000000002</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1626,6 +1678,9 @@
       <c r="T17" s="3" t="n">
         <v>0.096025</v>
       </c>
+      <c r="U17" s="3" t="n">
+        <v>0.09646249999999999</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1692,6 +1747,9 @@
       <c r="T18" s="3" t="n">
         <v>0.09619999999999999</v>
       </c>
+      <c r="U18" s="3" t="n">
+        <v>0.09677142857142859</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1758,6 +1816,9 @@
       <c r="T19" s="3" t="n">
         <v>0.09663749999999999</v>
       </c>
+      <c r="U19" s="3" t="n">
+        <v>0.0970125</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1824,6 +1885,9 @@
       <c r="T20" s="3" t="n">
         <v>0.09714444444444444</v>
       </c>
+      <c r="U20" s="3" t="n">
+        <v>0.09753333333333332</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1890,6 +1954,9 @@
       <c r="T21" s="3" t="n">
         <v>0.0968</v>
       </c>
+      <c r="U21" s="3" t="n">
+        <v>0.0975</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1956,6 +2023,9 @@
       <c r="T22" s="3" t="n">
         <v>0.09714</v>
       </c>
+      <c r="U22" s="3" t="n">
+        <v>0.09774000000000001</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2022,6 +2092,9 @@
       <c r="T23" s="3" t="n">
         <v>0.09803333333333335</v>
       </c>
+      <c r="U23" s="3" t="n">
+        <v>0.09794444444444445</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2088,6 +2161,9 @@
       <c r="T24" s="3" t="n">
         <v>0.09758</v>
       </c>
+      <c r="U24" s="3" t="n">
+        <v>0.09798</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2154,6 +2230,9 @@
       <c r="T25" s="3" t="n">
         <v>0.0985375</v>
       </c>
+      <c r="U25" s="3" t="n">
+        <v>0.0985375</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2220,6 +2299,9 @@
       <c r="T26" s="3" t="n">
         <v>0.098775</v>
       </c>
+      <c r="U26" s="3" t="n">
+        <v>0.09889999999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2286,6 +2368,9 @@
       <c r="T27" s="3" t="n">
         <v>0.09951111111111111</v>
       </c>
+      <c r="U27" s="3" t="n">
+        <v>0.09945555555555557</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2352,6 +2437,9 @@
       <c r="T28" s="3" t="n">
         <v>0.1000625</v>
       </c>
+      <c r="U28" s="3" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2418,6 +2506,9 @@
       <c r="T29" s="3" t="n">
         <v>0.1</v>
       </c>
+      <c r="U29" s="3" t="n">
+        <v>0.10025</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2484,6 +2575,9 @@
       <c r="T30" s="3" t="n">
         <v>0.1004428571428572</v>
       </c>
+      <c r="U30" s="3" t="n">
+        <v>0.1007285714285714</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2550,6 +2644,9 @@
       <c r="T31" s="3" t="n">
         <v>0.1006166666666666</v>
       </c>
+      <c r="U31" s="3" t="n">
+        <v>0.1012833333333333</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2616,6 +2713,9 @@
       <c r="T32" s="3" t="n">
         <v>0.1014285714285714</v>
       </c>
+      <c r="U32" s="3" t="n">
+        <v>0.1018571428571429</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2682,6 +2782,9 @@
       <c r="T33" s="3" t="n">
         <v>0.10175</v>
       </c>
+      <c r="U33" s="3" t="n">
+        <v>0.1021666666666667</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2748,6 +2851,9 @@
       <c r="T34" s="3" t="n">
         <v>0.102</v>
       </c>
+      <c r="U34" s="3" t="n">
+        <v>0.103</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2814,6 +2920,9 @@
       <c r="T35" s="3" t="n">
         <v>0.1043</v>
       </c>
+      <c r="U35" s="3" t="n">
+        <v>0.1053</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2880,6 +2989,9 @@
       <c r="T36" s="3" t="n">
         <v>0.1058333333333333</v>
       </c>
+      <c r="U36" s="3" t="n">
+        <v>0.107</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2946,6 +3058,9 @@
       <c r="T37" s="3" t="n">
         <v>0.1066</v>
       </c>
+      <c r="U37" s="3" t="n">
+        <v>0.1076</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3012,6 +3127,9 @@
       <c r="T38" s="3" t="n">
         <v>0.10746</v>
       </c>
+      <c r="U38" s="3" t="n">
+        <v>0.1078444444444445</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3078,6 +3196,9 @@
       <c r="T39" s="3" t="n">
         <v>0.10808</v>
       </c>
+      <c r="U39" s="3" t="n">
+        <v>0.10888</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3144,6 +3265,9 @@
       <c r="T40" s="3" t="n">
         <v>0.1092444444444444</v>
       </c>
+      <c r="U40" s="3" t="n">
+        <v>0.1094625</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3210,6 +3334,9 @@
       <c r="T41" s="3" t="n">
         <v>0.10876</v>
       </c>
+      <c r="U41" s="3" t="n">
+        <v>0.1094666666666667</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3276,6 +3403,9 @@
       <c r="T42" s="3" t="n">
         <v>0.1095</v>
       </c>
+      <c r="U42" s="3" t="n">
+        <v>0.1099375</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3342,6 +3472,9 @@
       <c r="T43" s="3" t="n">
         <v>0.10942</v>
       </c>
+      <c r="U43" s="3" t="n">
+        <v>0.11052</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3408,6 +3541,9 @@
       <c r="T44" s="3" t="n">
         <v>0.1106375</v>
       </c>
+      <c r="U44" s="3" t="n">
+        <v>0.110875</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3474,6 +3610,9 @@
       <c r="T45" s="3" t="n">
         <v>0.1102333333333333</v>
       </c>
+      <c r="U45" s="3" t="n">
+        <v>0.1108833333333333</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3540,6 +3679,9 @@
       <c r="T46" s="3" t="n">
         <v>0.1108</v>
       </c>
+      <c r="U46" s="3" t="n">
+        <v>0.1118</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3606,6 +3748,9 @@
       <c r="T47" s="3" t="n">
         <v>0.1114142857142857</v>
       </c>
+      <c r="U47" s="3" t="n">
+        <v>0.1120285714285714</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3672,6 +3817,9 @@
       <c r="T48" s="3" t="n">
         <v>0.111</v>
       </c>
+      <c r="U48" s="3" t="n">
+        <v>0.1119166666666667</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3738,6 +3886,9 @@
       <c r="T49" s="3" t="n">
         <v>0.1115833333333333</v>
       </c>
+      <c r="U49" s="3" t="n">
+        <v>0.1124166666666667</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3804,6 +3955,9 @@
       <c r="T50" s="3" t="n">
         <v>0.1116</v>
       </c>
+      <c r="U50" s="3" t="n">
+        <v>0.1128333333333333</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3870,6 +4024,9 @@
       <c r="T51" s="3" t="n">
         <v>0.112625</v>
       </c>
+      <c r="U51" s="3" t="n">
+        <v>0.11425</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3936,6 +4093,9 @@
       <c r="T52" s="3" t="n">
         <v>0.1135</v>
       </c>
+      <c r="U52" s="3" t="n">
+        <v>0.11475</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4002,6 +4162,9 @@
       <c r="T53" s="3" t="n">
         <v>0.114</v>
       </c>
+      <c r="U53" s="3" t="n">
+        <v>0.115625</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4068,6 +4231,9 @@
       <c r="T54" s="3" t="n">
         <v>0.1145</v>
       </c>
+      <c r="U54" s="3" t="n">
+        <v>0.1153333333333333</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4133,6 +4299,42 @@
       </c>
       <c r="T55" s="3" t="n">
         <v>0.1165</v>
+      </c>
+      <c r="U55" s="3" t="n">
+        <v>0.116</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>10.002030A</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>01-Aug-2030</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="n"/>
+      <c r="D56" s="4" t="n"/>
+      <c r="E56" s="4" t="n"/>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
+      <c r="I56" s="4" t="n"/>
+      <c r="J56" s="4" t="n"/>
+      <c r="K56" s="4" t="n"/>
+      <c r="L56" s="4" t="n"/>
+      <c r="M56" s="4" t="n"/>
+      <c r="N56" s="4" t="n"/>
+      <c r="O56" s="4" t="n"/>
+      <c r="P56" s="4" t="n"/>
+      <c r="Q56" s="4" t="n"/>
+      <c r="R56" s="4" t="n"/>
+      <c r="S56" s="4" t="n"/>
+      <c r="T56" s="4" t="n"/>
+      <c r="U56" s="3" t="n">
+        <v>0.10098</v>
       </c>
     </row>
   </sheetData>
@@ -4146,7 +4348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T40"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4169,6 +4371,7 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4272,6 +4475,11 @@
           <t>11-May-26</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>12-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4338,6 +4546,9 @@
       <c r="T2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4404,6 +4615,9 @@
       <c r="T3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="U3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4470,6 +4684,9 @@
       <c r="T4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4536,6 +4753,9 @@
       <c r="T5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="U5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4602,6 +4822,9 @@
       <c r="T6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4668,6 +4891,9 @@
       <c r="T7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4734,6 +4960,9 @@
       <c r="T8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4800,6 +5029,9 @@
       <c r="T9" s="3" t="n">
         <v>0.1444</v>
       </c>
+      <c r="U9" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4866,6 +5098,9 @@
       <c r="T10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4932,6 +5167,9 @@
       <c r="T11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4998,6 +5236,9 @@
       <c r="T12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5064,6 +5305,9 @@
       <c r="T13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5130,6 +5374,9 @@
       <c r="T14" s="3" t="n">
         <v>0.1454</v>
       </c>
+      <c r="U14" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5196,6 +5443,9 @@
       <c r="T15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5262,6 +5512,9 @@
       <c r="T16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5328,6 +5581,9 @@
       <c r="T17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5394,6 +5650,9 @@
       <c r="T18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5460,6 +5719,9 @@
       <c r="T19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5526,6 +5788,9 @@
       <c r="T20" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U20" s="3" t="n">
+        <v>0.08666666666666667</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5592,6 +5857,9 @@
       <c r="T21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5658,6 +5926,9 @@
       <c r="T22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5724,6 +5995,9 @@
       <c r="T23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5790,6 +6064,9 @@
       <c r="T24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -5856,6 +6133,9 @@
       <c r="T25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -5922,6 +6202,9 @@
       <c r="T26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5988,6 +6271,9 @@
       <c r="T27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -6054,6 +6340,9 @@
       <c r="T28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -6120,6 +6409,9 @@
       <c r="T29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -6186,6 +6478,9 @@
       <c r="T30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -6252,6 +6547,9 @@
       <c r="T31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -6318,6 +6616,9 @@
       <c r="T32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6384,6 +6685,9 @@
       <c r="T33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6450,6 +6754,9 @@
       <c r="T34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6516,6 +6823,9 @@
       <c r="T35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6582,6 +6892,9 @@
       <c r="T36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6648,6 +6961,9 @@
       <c r="T37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6714,6 +7030,9 @@
       <c r="T38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6780,6 +7099,9 @@
       <c r="T39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="U39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6844,6 +7166,9 @@
         <v>0.13</v>
       </c>
       <c r="T40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="U40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update treasury bond yields - 2026-05-14
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U56"/>
+  <dimension ref="A1:V56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -469,6 +469,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -577,6 +578,11 @@
           <t>12-May-26</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>13-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -646,6 +652,9 @@
       <c r="U2" s="3" t="n">
         <v>0.08028333333333335</v>
       </c>
+      <c r="V2" s="3" t="n">
+        <v>0.08028333333333335</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -715,6 +724,9 @@
       <c r="U3" s="3" t="n">
         <v>0.08130000000000001</v>
       </c>
+      <c r="V3" s="3" t="n">
+        <v>0.08130000000000001</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -784,6 +796,9 @@
       <c r="U4" s="3" t="n">
         <v>0.08259999999999999</v>
       </c>
+      <c r="V4" s="3" t="n">
+        <v>0.08259999999999999</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -853,6 +868,9 @@
       <c r="U5" s="3" t="n">
         <v>0.08415555555555555</v>
       </c>
+      <c r="V5" s="3" t="n">
+        <v>0.08410000000000001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -922,6 +940,9 @@
       <c r="U6" s="3" t="n">
         <v>0.08448</v>
       </c>
+      <c r="V6" s="3" t="n">
+        <v>0.08448</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -991,6 +1012,9 @@
       <c r="U7" s="3" t="n">
         <v>0.08642857142857142</v>
       </c>
+      <c r="V7" s="3" t="n">
+        <v>0.08642857142857142</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1060,6 +1084,9 @@
       <c r="U8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="V8" s="3" t="n">
+        <v>0.08629999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1129,6 +1156,9 @@
       <c r="U9" s="3" t="n">
         <v>0.08882</v>
       </c>
+      <c r="V9" s="3" t="n">
+        <v>0.08882</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1198,6 +1228,9 @@
       <c r="U10" s="3" t="n">
         <v>0.0898</v>
       </c>
+      <c r="V10" s="3" t="n">
+        <v>0.0898</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1267,6 +1300,9 @@
       <c r="U11" s="3" t="n">
         <v>0.09014</v>
       </c>
+      <c r="V11" s="3" t="n">
+        <v>0.09014</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1336,6 +1372,9 @@
       <c r="U12" s="3" t="n">
         <v>0.09144999999999999</v>
       </c>
+      <c r="V12" s="3" t="n">
+        <v>0.09144999999999999</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1405,6 +1444,9 @@
       <c r="U13" s="3" t="n">
         <v>0.09346666666666666</v>
       </c>
+      <c r="V13" s="3" t="n">
+        <v>0.09346666666666666</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1474,6 +1516,9 @@
       <c r="U14" s="3" t="n">
         <v>0.09514444444444443</v>
       </c>
+      <c r="V14" s="3" t="n">
+        <v>0.09536666666666667</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1543,6 +1588,9 @@
       <c r="U15" s="3" t="n">
         <v>0.0949857142857143</v>
       </c>
+      <c r="V15" s="3" t="n">
+        <v>0.09520000000000002</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1612,6 +1660,9 @@
       <c r="U16" s="3" t="n">
         <v>0.09612500000000002</v>
       </c>
+      <c r="V16" s="3" t="n">
+        <v>0.09625</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1681,6 +1732,9 @@
       <c r="U17" s="3" t="n">
         <v>0.09646249999999999</v>
       </c>
+      <c r="V17" s="3" t="n">
+        <v>0.09658750000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1750,6 +1804,9 @@
       <c r="U18" s="3" t="n">
         <v>0.09677142857142859</v>
       </c>
+      <c r="V18" s="3" t="n">
+        <v>0.09684285714285715</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1819,6 +1876,9 @@
       <c r="U19" s="3" t="n">
         <v>0.0970125</v>
       </c>
+      <c r="V19" s="3" t="n">
+        <v>0.09719999999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1888,6 +1948,9 @@
       <c r="U20" s="3" t="n">
         <v>0.09753333333333332</v>
       </c>
+      <c r="V20" s="3" t="n">
+        <v>0.09758888888888889</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1957,6 +2020,9 @@
       <c r="U21" s="3" t="n">
         <v>0.0975</v>
       </c>
+      <c r="V21" s="3" t="n">
+        <v>0.0975</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2026,6 +2092,9 @@
       <c r="U22" s="3" t="n">
         <v>0.09774000000000001</v>
       </c>
+      <c r="V22" s="3" t="n">
+        <v>0.09774000000000001</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2095,6 +2164,9 @@
       <c r="U23" s="3" t="n">
         <v>0.09794444444444445</v>
       </c>
+      <c r="V23" s="3" t="n">
+        <v>0.09811111111111112</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2164,6 +2236,9 @@
       <c r="U24" s="3" t="n">
         <v>0.09798</v>
       </c>
+      <c r="V24" s="3" t="n">
+        <v>0.09808000000000001</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2233,6 +2308,9 @@
       <c r="U25" s="3" t="n">
         <v>0.0985375</v>
       </c>
+      <c r="V25" s="3" t="n">
+        <v>0.09872499999999999</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2302,6 +2380,9 @@
       <c r="U26" s="3" t="n">
         <v>0.09889999999999999</v>
       </c>
+      <c r="V26" s="3" t="n">
+        <v>0.09896249999999998</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2371,6 +2452,9 @@
       <c r="U27" s="3" t="n">
         <v>0.09945555555555557</v>
       </c>
+      <c r="V27" s="3" t="n">
+        <v>0.09956666666666669</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2440,6 +2524,9 @@
       <c r="U28" s="3" t="n">
         <v>0.1</v>
       </c>
+      <c r="V28" s="3" t="n">
+        <v>0.1000625</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2509,6 +2596,9 @@
       <c r="U29" s="3" t="n">
         <v>0.10025</v>
       </c>
+      <c r="V29" s="3" t="n">
+        <v>0.1001666666666667</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2578,6 +2668,9 @@
       <c r="U30" s="3" t="n">
         <v>0.1007285714285714</v>
       </c>
+      <c r="V30" s="3" t="n">
+        <v>0.1005857142857143</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2647,6 +2740,9 @@
       <c r="U31" s="3" t="n">
         <v>0.1012833333333333</v>
       </c>
+      <c r="V31" s="3" t="n">
+        <v>0.1012</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2716,6 +2812,9 @@
       <c r="U32" s="3" t="n">
         <v>0.1018571428571429</v>
       </c>
+      <c r="V32" s="3" t="n">
+        <v>0.1018571428571429</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2785,6 +2884,9 @@
       <c r="U33" s="3" t="n">
         <v>0.1021666666666667</v>
       </c>
+      <c r="V33" s="3" t="n">
+        <v>0.1021666666666667</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2854,6 +2956,9 @@
       <c r="U34" s="3" t="n">
         <v>0.103</v>
       </c>
+      <c r="V34" s="3" t="n">
+        <v>0.103</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2923,6 +3028,9 @@
       <c r="U35" s="3" t="n">
         <v>0.1053</v>
       </c>
+      <c r="V35" s="3" t="n">
+        <v>0.1053</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2992,6 +3100,9 @@
       <c r="U36" s="3" t="n">
         <v>0.107</v>
       </c>
+      <c r="V36" s="3" t="n">
+        <v>0.107</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3061,6 +3172,9 @@
       <c r="U37" s="3" t="n">
         <v>0.1076</v>
       </c>
+      <c r="V37" s="3" t="n">
+        <v>0.1076625</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3130,6 +3244,9 @@
       <c r="U38" s="3" t="n">
         <v>0.1078444444444445</v>
       </c>
+      <c r="V38" s="3" t="n">
+        <v>0.107825</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3199,6 +3316,9 @@
       <c r="U39" s="3" t="n">
         <v>0.10888</v>
       </c>
+      <c r="V39" s="3" t="n">
+        <v>0.10888</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3268,6 +3388,9 @@
       <c r="U40" s="3" t="n">
         <v>0.1094625</v>
       </c>
+      <c r="V40" s="3" t="n">
+        <v>0.1094625</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3337,6 +3460,9 @@
       <c r="U41" s="3" t="n">
         <v>0.1094666666666667</v>
       </c>
+      <c r="V41" s="3" t="n">
+        <v>0.1094666666666667</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3406,6 +3532,9 @@
       <c r="U42" s="3" t="n">
         <v>0.1099375</v>
       </c>
+      <c r="V42" s="3" t="n">
+        <v>0.1098125</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3475,6 +3604,9 @@
       <c r="U43" s="3" t="n">
         <v>0.11052</v>
       </c>
+      <c r="V43" s="3" t="n">
+        <v>0.11052</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3544,6 +3676,9 @@
       <c r="U44" s="3" t="n">
         <v>0.110875</v>
       </c>
+      <c r="V44" s="3" t="n">
+        <v>0.111125</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3613,6 +3748,9 @@
       <c r="U45" s="3" t="n">
         <v>0.1108833333333333</v>
       </c>
+      <c r="V45" s="3" t="n">
+        <v>0.1109333333333333</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3682,6 +3820,9 @@
       <c r="U46" s="3" t="n">
         <v>0.1118</v>
       </c>
+      <c r="V46" s="3" t="n">
+        <v>0.1118</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3751,6 +3892,9 @@
       <c r="U47" s="3" t="n">
         <v>0.1120285714285714</v>
       </c>
+      <c r="V47" s="3" t="n">
+        <v>0.1121</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3820,6 +3964,9 @@
       <c r="U48" s="3" t="n">
         <v>0.1119166666666667</v>
       </c>
+      <c r="V48" s="3" t="n">
+        <v>0.1120833333333333</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3889,6 +4036,9 @@
       <c r="U49" s="3" t="n">
         <v>0.1124166666666667</v>
       </c>
+      <c r="V49" s="3" t="n">
+        <v>0.1124166666666667</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3958,6 +4108,9 @@
       <c r="U50" s="3" t="n">
         <v>0.1128333333333333</v>
       </c>
+      <c r="V50" s="3" t="n">
+        <v>0.1129285714285714</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4027,6 +4180,9 @@
       <c r="U51" s="3" t="n">
         <v>0.11425</v>
       </c>
+      <c r="V51" s="3" t="n">
+        <v>0.11425</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4096,6 +4252,9 @@
       <c r="U52" s="3" t="n">
         <v>0.11475</v>
       </c>
+      <c r="V52" s="3" t="n">
+        <v>0.11475</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4165,6 +4324,9 @@
       <c r="U53" s="3" t="n">
         <v>0.115625</v>
       </c>
+      <c r="V53" s="3" t="n">
+        <v>0.115625</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4234,6 +4396,9 @@
       <c r="U54" s="3" t="n">
         <v>0.1153333333333333</v>
       </c>
+      <c r="V54" s="3" t="n">
+        <v>0.1153333333333333</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4301,6 +4466,9 @@
         <v>0.1165</v>
       </c>
       <c r="U55" s="3" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="V55" s="3" t="n">
         <v>0.116</v>
       </c>
     </row>
@@ -4336,6 +4504,9 @@
       <c r="U56" s="3" t="n">
         <v>0.10098</v>
       </c>
+      <c r="V56" s="3" t="n">
+        <v>0.10088</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4348,7 +4519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U40"/>
+  <dimension ref="A1:V40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4372,6 +4543,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4480,6 +4652,11 @@
           <t>12-May-26</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>13-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4549,6 +4726,9 @@
       <c r="U2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4618,6 +4798,9 @@
       <c r="U3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="V3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4687,6 +4870,9 @@
       <c r="U4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4756,6 +4942,9 @@
       <c r="U5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="V5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4825,6 +5014,9 @@
       <c r="U6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4894,6 +5086,9 @@
       <c r="U7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4963,6 +5158,9 @@
       <c r="U8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -5032,6 +5230,9 @@
       <c r="U9" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V9" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -5101,6 +5302,9 @@
       <c r="U10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -5170,6 +5374,9 @@
       <c r="U11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5239,6 +5446,9 @@
       <c r="U12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5308,6 +5518,9 @@
       <c r="U13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5377,6 +5590,9 @@
       <c r="U14" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V14" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5446,6 +5662,9 @@
       <c r="U15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5515,6 +5734,9 @@
       <c r="U16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5584,6 +5806,9 @@
       <c r="U17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5653,6 +5878,9 @@
       <c r="U18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5722,6 +5950,9 @@
       <c r="U19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5791,6 +6022,9 @@
       <c r="U20" s="3" t="n">
         <v>0.08666666666666667</v>
       </c>
+      <c r="V20" s="3" t="n">
+        <v>0.08666666666666667</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5860,6 +6094,9 @@
       <c r="U21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5929,6 +6166,9 @@
       <c r="U22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5998,6 +6238,9 @@
       <c r="U23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6067,6 +6310,9 @@
       <c r="U24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6136,6 +6382,9 @@
       <c r="U25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6205,6 +6454,9 @@
       <c r="U26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6274,6 +6526,9 @@
       <c r="U27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -6343,6 +6598,9 @@
       <c r="U28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -6412,6 +6670,9 @@
       <c r="U29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -6481,6 +6742,9 @@
       <c r="U30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -6550,6 +6814,9 @@
       <c r="U31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -6619,6 +6886,9 @@
       <c r="U32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6688,6 +6958,9 @@
       <c r="U33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6757,6 +7030,9 @@
       <c r="U34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6826,6 +7102,9 @@
       <c r="U35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6895,6 +7174,9 @@
       <c r="U36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6964,6 +7246,9 @@
       <c r="U37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -7033,6 +7318,9 @@
       <c r="U38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7102,6 +7390,9 @@
       <c r="U39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="V39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7169,6 +7460,9 @@
         <v>0.13</v>
       </c>
       <c r="U40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="V40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update treasury bond yields - 2026-05-15
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V56"/>
+  <dimension ref="A1:W56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,6 +470,7 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -583,6 +584,11 @@
           <t>13-May-26</t>
         </is>
       </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>14-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -727,6 +733,9 @@
       <c r="V3" s="3" t="n">
         <v>0.08130000000000001</v>
       </c>
+      <c r="W3" s="3" t="n">
+        <v>0.08121666666666667</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -799,6 +808,9 @@
       <c r="V4" s="3" t="n">
         <v>0.08259999999999999</v>
       </c>
+      <c r="W4" s="3" t="n">
+        <v>0.08259999999999999</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -871,6 +883,9 @@
       <c r="V5" s="3" t="n">
         <v>0.08410000000000001</v>
       </c>
+      <c r="W5" s="3" t="n">
+        <v>0.08365555555555555</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -943,6 +958,9 @@
       <c r="V6" s="3" t="n">
         <v>0.08448</v>
       </c>
+      <c r="W6" s="3" t="n">
+        <v>0.08427999999999999</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1015,6 +1033,9 @@
       <c r="V7" s="3" t="n">
         <v>0.08642857142857142</v>
       </c>
+      <c r="W7" s="3" t="n">
+        <v>0.08650000000000001</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1087,6 +1108,9 @@
       <c r="V8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="W8" s="3" t="n">
+        <v>0.08629999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1159,6 +1183,9 @@
       <c r="V9" s="3" t="n">
         <v>0.08882</v>
       </c>
+      <c r="W9" s="3" t="n">
+        <v>0.08851999999999999</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1231,6 +1258,9 @@
       <c r="V10" s="3" t="n">
         <v>0.0898</v>
       </c>
+      <c r="W10" s="3" t="n">
+        <v>0.08965714285714287</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1303,6 +1333,9 @@
       <c r="V11" s="3" t="n">
         <v>0.09014</v>
       </c>
+      <c r="W11" s="3" t="n">
+        <v>0.08984</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1375,6 +1408,9 @@
       <c r="V12" s="3" t="n">
         <v>0.09144999999999999</v>
       </c>
+      <c r="W12" s="3" t="n">
+        <v>0.09103333333333334</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1447,6 +1483,9 @@
       <c r="V13" s="3" t="n">
         <v>0.09346666666666666</v>
       </c>
+      <c r="W13" s="3" t="n">
+        <v>0.09329999999999999</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1519,6 +1558,9 @@
       <c r="V14" s="3" t="n">
         <v>0.09536666666666667</v>
       </c>
+      <c r="W14" s="3" t="n">
+        <v>0.09536666666666666</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1591,6 +1633,9 @@
       <c r="V15" s="3" t="n">
         <v>0.09520000000000002</v>
       </c>
+      <c r="W15" s="3" t="n">
+        <v>0.09519999999999999</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1663,6 +1708,9 @@
       <c r="V16" s="3" t="n">
         <v>0.09625</v>
       </c>
+      <c r="W16" s="3" t="n">
+        <v>0.09625</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1735,6 +1783,9 @@
       <c r="V17" s="3" t="n">
         <v>0.09658750000000001</v>
       </c>
+      <c r="W17" s="3" t="n">
+        <v>0.09658750000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1807,6 +1858,9 @@
       <c r="V18" s="3" t="n">
         <v>0.09684285714285715</v>
       </c>
+      <c r="W18" s="3" t="n">
+        <v>0.09691428571428572</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1879,6 +1933,9 @@
       <c r="V19" s="3" t="n">
         <v>0.09719999999999999</v>
       </c>
+      <c r="W19" s="3" t="n">
+        <v>0.09720000000000001</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1951,6 +2008,9 @@
       <c r="V20" s="3" t="n">
         <v>0.09758888888888889</v>
       </c>
+      <c r="W20" s="3" t="n">
+        <v>0.09764444444444446</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2023,6 +2083,9 @@
       <c r="V21" s="3" t="n">
         <v>0.0975</v>
       </c>
+      <c r="W21" s="3" t="n">
+        <v>0.0974</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2095,6 +2158,9 @@
       <c r="V22" s="3" t="n">
         <v>0.09774000000000001</v>
       </c>
+      <c r="W22" s="3" t="n">
+        <v>0.09774000000000001</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2167,6 +2233,9 @@
       <c r="V23" s="3" t="n">
         <v>0.09811111111111112</v>
       </c>
+      <c r="W23" s="3" t="n">
+        <v>0.0983888888888889</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2239,6 +2308,9 @@
       <c r="V24" s="3" t="n">
         <v>0.09808000000000001</v>
       </c>
+      <c r="W24" s="3" t="n">
+        <v>0.09798000000000003</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2311,6 +2383,9 @@
       <c r="V25" s="3" t="n">
         <v>0.09872499999999999</v>
       </c>
+      <c r="W25" s="3" t="n">
+        <v>0.09909999999999999</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2383,6 +2458,9 @@
       <c r="V26" s="3" t="n">
         <v>0.09896249999999998</v>
       </c>
+      <c r="W26" s="3" t="n">
+        <v>0.09927499999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2455,6 +2533,9 @@
       <c r="V27" s="3" t="n">
         <v>0.09956666666666669</v>
       </c>
+      <c r="W27" s="3" t="n">
+        <v>0.09984444444444446</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2527,6 +2608,9 @@
       <c r="V28" s="3" t="n">
         <v>0.1000625</v>
       </c>
+      <c r="W28" s="3" t="n">
+        <v>0.1000625</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2599,6 +2683,9 @@
       <c r="V29" s="3" t="n">
         <v>0.1001666666666667</v>
       </c>
+      <c r="W29" s="3" t="n">
+        <v>0.10025</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2671,6 +2758,9 @@
       <c r="V30" s="3" t="n">
         <v>0.1005857142857143</v>
       </c>
+      <c r="W30" s="3" t="n">
+        <v>0.1006571428571429</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2743,6 +2833,9 @@
       <c r="V31" s="3" t="n">
         <v>0.1012</v>
       </c>
+      <c r="W31" s="3" t="n">
+        <v>0.1012</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2815,6 +2908,9 @@
       <c r="V32" s="3" t="n">
         <v>0.1018571428571429</v>
       </c>
+      <c r="W32" s="3" t="n">
+        <v>0.1018571428571429</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2887,6 +2983,9 @@
       <c r="V33" s="3" t="n">
         <v>0.1021666666666667</v>
       </c>
+      <c r="W33" s="3" t="n">
+        <v>0.1021666666666667</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2959,6 +3058,9 @@
       <c r="V34" s="3" t="n">
         <v>0.103</v>
       </c>
+      <c r="W34" s="3" t="n">
+        <v>0.1027</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3031,6 +3133,9 @@
       <c r="V35" s="3" t="n">
         <v>0.1053</v>
       </c>
+      <c r="W35" s="3" t="n">
+        <v>0.1052</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3103,6 +3208,9 @@
       <c r="V36" s="3" t="n">
         <v>0.107</v>
       </c>
+      <c r="W36" s="3" t="n">
+        <v>0.10675</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3175,6 +3283,9 @@
       <c r="V37" s="3" t="n">
         <v>0.1076625</v>
       </c>
+      <c r="W37" s="3" t="n">
+        <v>0.1074125</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3247,6 +3358,9 @@
       <c r="V38" s="3" t="n">
         <v>0.107825</v>
       </c>
+      <c r="W38" s="3" t="n">
+        <v>0.1076777777777778</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3319,6 +3433,9 @@
       <c r="V39" s="3" t="n">
         <v>0.10888</v>
       </c>
+      <c r="W39" s="3" t="n">
+        <v>0.10888</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3391,6 +3508,9 @@
       <c r="V40" s="3" t="n">
         <v>0.1094625</v>
       </c>
+      <c r="W40" s="3" t="n">
+        <v>0.1094625</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3463,6 +3583,9 @@
       <c r="V41" s="3" t="n">
         <v>0.1094666666666667</v>
       </c>
+      <c r="W41" s="3" t="n">
+        <v>0.1093833333333333</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3535,6 +3658,9 @@
       <c r="V42" s="3" t="n">
         <v>0.1098125</v>
       </c>
+      <c r="W42" s="3" t="n">
+        <v>0.1098125</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3607,6 +3733,9 @@
       <c r="V43" s="3" t="n">
         <v>0.11052</v>
       </c>
+      <c r="W43" s="3" t="n">
+        <v>0.11042</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3679,6 +3808,9 @@
       <c r="V44" s="3" t="n">
         <v>0.111125</v>
       </c>
+      <c r="W44" s="3" t="n">
+        <v>0.1112555555555556</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3751,6 +3883,9 @@
       <c r="V45" s="3" t="n">
         <v>0.1109333333333333</v>
       </c>
+      <c r="W45" s="3" t="n">
+        <v>0.1109</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3823,6 +3958,9 @@
       <c r="V46" s="3" t="n">
         <v>0.1118</v>
       </c>
+      <c r="W46" s="3" t="n">
+        <v>0.11174</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3895,6 +4033,9 @@
       <c r="V47" s="3" t="n">
         <v>0.1121</v>
       </c>
+      <c r="W47" s="3" t="n">
+        <v>0.1121</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3967,6 +4108,9 @@
       <c r="V48" s="3" t="n">
         <v>0.1120833333333333</v>
       </c>
+      <c r="W48" s="3" t="n">
+        <v>0.1122857142857143</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4039,6 +4183,9 @@
       <c r="V49" s="3" t="n">
         <v>0.1124166666666667</v>
       </c>
+      <c r="W49" s="3" t="n">
+        <v>0.1124166666666667</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4111,6 +4258,9 @@
       <c r="V50" s="3" t="n">
         <v>0.1129285714285714</v>
       </c>
+      <c r="W50" s="3" t="n">
+        <v>0.1127857142857143</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4183,6 +4333,9 @@
       <c r="V51" s="3" t="n">
         <v>0.11425</v>
       </c>
+      <c r="W51" s="3" t="n">
+        <v>0.114</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4255,6 +4408,9 @@
       <c r="V52" s="3" t="n">
         <v>0.11475</v>
       </c>
+      <c r="W52" s="3" t="n">
+        <v>0.1145</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4327,6 +4483,9 @@
       <c r="V53" s="3" t="n">
         <v>0.115625</v>
       </c>
+      <c r="W53" s="3" t="n">
+        <v>0.115</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4399,6 +4558,9 @@
       <c r="V54" s="3" t="n">
         <v>0.1153333333333333</v>
       </c>
+      <c r="W54" s="3" t="n">
+        <v>0.115875</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4470,6 +4632,9 @@
       </c>
       <c r="V55" s="3" t="n">
         <v>0.116</v>
+      </c>
+      <c r="W55" s="3" t="n">
+        <v>0.1166666666666667</v>
       </c>
     </row>
     <row r="56">
@@ -4507,6 +4672,9 @@
       <c r="V56" s="3" t="n">
         <v>0.10088</v>
       </c>
+      <c r="W56" s="3" t="n">
+        <v>0.1009833333333334</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4519,7 +4687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V40"/>
+  <dimension ref="A1:W40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4544,6 +4712,7 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4657,6 +4826,11 @@
           <t>13-May-26</t>
         </is>
       </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>14-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4729,6 +4903,9 @@
       <c r="V2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4801,6 +4978,9 @@
       <c r="V3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="W3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4873,6 +5053,9 @@
       <c r="V4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4945,6 +5128,9 @@
       <c r="V5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="W5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -5017,6 +5203,9 @@
       <c r="V6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -5089,6 +5278,9 @@
       <c r="V7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -5161,6 +5353,9 @@
       <c r="V8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -5233,6 +5428,9 @@
       <c r="V9" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W9" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -5305,6 +5503,9 @@
       <c r="V10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -5377,6 +5578,9 @@
       <c r="V11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5449,6 +5653,9 @@
       <c r="V12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5521,6 +5728,9 @@
       <c r="V13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5593,6 +5803,9 @@
       <c r="V14" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W14" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5665,6 +5878,9 @@
       <c r="V15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5737,6 +5953,9 @@
       <c r="V16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5809,6 +6028,9 @@
       <c r="V17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5881,6 +6103,9 @@
       <c r="V18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5953,6 +6178,9 @@
       <c r="V19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6025,6 +6253,9 @@
       <c r="V20" s="3" t="n">
         <v>0.08666666666666667</v>
       </c>
+      <c r="W20" s="3" t="n">
+        <v>0.08666666666666667</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6097,6 +6328,9 @@
       <c r="V21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6169,6 +6403,9 @@
       <c r="V22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6241,6 +6478,9 @@
       <c r="V23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6313,6 +6553,9 @@
       <c r="V24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6385,6 +6628,9 @@
       <c r="V25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6457,6 +6703,9 @@
       <c r="V26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6529,6 +6778,9 @@
       <c r="V27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -6601,6 +6853,9 @@
       <c r="V28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -6673,6 +6928,9 @@
       <c r="V29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -6745,6 +7003,9 @@
       <c r="V30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -6817,6 +7078,9 @@
       <c r="V31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -6889,6 +7153,9 @@
       <c r="V32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6961,6 +7228,9 @@
       <c r="V33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -7033,6 +7303,9 @@
       <c r="V34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -7105,6 +7378,9 @@
       <c r="V35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -7177,6 +7453,9 @@
       <c r="V36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -7249,6 +7528,9 @@
       <c r="V37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -7321,6 +7603,9 @@
       <c r="V38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7393,6 +7678,9 @@
       <c r="V39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="W39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7463,6 +7751,9 @@
         <v>0.13</v>
       </c>
       <c r="V40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="W40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update treasury bond yields - 2026-05-19
</commit_message>
<xml_diff>
--- a/output/treasury_bond_yields.xlsx
+++ b/output/treasury_bond_yields.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W56"/>
+  <dimension ref="A1:X56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -471,6 +471,7 @@
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,6 +590,11 @@
           <t>14-May-26</t>
         </is>
       </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>18-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -736,6 +742,9 @@
       <c r="W3" s="3" t="n">
         <v>0.08121666666666667</v>
       </c>
+      <c r="X3" s="3" t="n">
+        <v>0.08038333333333335</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -811,6 +820,9 @@
       <c r="W4" s="3" t="n">
         <v>0.08259999999999999</v>
       </c>
+      <c r="X4" s="3" t="n">
+        <v>0.08278749999999999</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -886,6 +898,9 @@
       <c r="W5" s="3" t="n">
         <v>0.08365555555555555</v>
       </c>
+      <c r="X5" s="3" t="n">
+        <v>0.08348888888888889</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -961,6 +976,9 @@
       <c r="W6" s="3" t="n">
         <v>0.08427999999999999</v>
       </c>
+      <c r="X6" s="3" t="n">
+        <v>0.08418</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1036,6 +1054,9 @@
       <c r="W7" s="3" t="n">
         <v>0.08650000000000001</v>
       </c>
+      <c r="X7" s="3" t="n">
+        <v>0.08599999999999999</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1111,6 +1132,9 @@
       <c r="W8" s="3" t="n">
         <v>0.08629999999999999</v>
       </c>
+      <c r="X8" s="3" t="n">
+        <v>0.08649999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1186,6 +1210,9 @@
       <c r="W9" s="3" t="n">
         <v>0.08851999999999999</v>
       </c>
+      <c r="X9" s="3" t="n">
+        <v>0.08831999999999998</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1261,6 +1288,9 @@
       <c r="W10" s="3" t="n">
         <v>0.08965714285714287</v>
       </c>
+      <c r="X10" s="3" t="n">
+        <v>0.08979999999999999</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1336,6 +1366,9 @@
       <c r="W11" s="3" t="n">
         <v>0.08984</v>
       </c>
+      <c r="X11" s="3" t="n">
+        <v>0.08993999999999999</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1411,6 +1444,9 @@
       <c r="W12" s="3" t="n">
         <v>0.09103333333333334</v>
       </c>
+      <c r="X12" s="3" t="n">
+        <v>0.09103333333333334</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1486,6 +1522,9 @@
       <c r="W13" s="3" t="n">
         <v>0.09329999999999999</v>
       </c>
+      <c r="X13" s="3" t="n">
+        <v>0.09296666666666666</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1561,6 +1600,9 @@
       <c r="W14" s="3" t="n">
         <v>0.09536666666666666</v>
       </c>
+      <c r="X14" s="3" t="n">
+        <v>0.09564444444444446</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1636,6 +1678,9 @@
       <c r="W15" s="3" t="n">
         <v>0.09519999999999999</v>
       </c>
+      <c r="X15" s="3" t="n">
+        <v>0.09555714285714287</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1711,6 +1756,9 @@
       <c r="W16" s="3" t="n">
         <v>0.09625</v>
       </c>
+      <c r="X16" s="3" t="n">
+        <v>0.0965625</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1786,6 +1834,9 @@
       <c r="W17" s="3" t="n">
         <v>0.09658750000000001</v>
       </c>
+      <c r="X17" s="3" t="n">
+        <v>0.09702500000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1861,6 +1912,9 @@
       <c r="W18" s="3" t="n">
         <v>0.09691428571428572</v>
       </c>
+      <c r="X18" s="3" t="n">
+        <v>0.09719999999999998</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1936,6 +1990,9 @@
       <c r="W19" s="3" t="n">
         <v>0.09720000000000001</v>
       </c>
+      <c r="X19" s="3" t="n">
+        <v>0.097575</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2011,6 +2068,9 @@
       <c r="W20" s="3" t="n">
         <v>0.09764444444444446</v>
       </c>
+      <c r="X20" s="3" t="n">
+        <v>0.09792222222222222</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2086,6 +2146,9 @@
       <c r="W21" s="3" t="n">
         <v>0.0974</v>
       </c>
+      <c r="X21" s="3" t="n">
+        <v>0.09769999999999998</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2161,6 +2224,9 @@
       <c r="W22" s="3" t="n">
         <v>0.09774000000000001</v>
       </c>
+      <c r="X22" s="3" t="n">
+        <v>0.09784000000000001</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2236,6 +2302,9 @@
       <c r="W23" s="3" t="n">
         <v>0.0983888888888889</v>
       </c>
+      <c r="X23" s="3" t="n">
+        <v>0.09877777777777778</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2311,6 +2380,9 @@
       <c r="W24" s="3" t="n">
         <v>0.09798000000000003</v>
       </c>
+      <c r="X24" s="3" t="n">
+        <v>0.09808000000000001</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2386,6 +2458,9 @@
       <c r="W25" s="3" t="n">
         <v>0.09909999999999999</v>
       </c>
+      <c r="X25" s="3" t="n">
+        <v>0.09935000000000001</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2461,6 +2536,9 @@
       <c r="W26" s="3" t="n">
         <v>0.09927499999999999</v>
       </c>
+      <c r="X26" s="3" t="n">
+        <v>0.09958750000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2536,6 +2614,9 @@
       <c r="W27" s="3" t="n">
         <v>0.09984444444444446</v>
       </c>
+      <c r="X27" s="3" t="n">
+        <v>0.1000666666666667</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2611,6 +2692,9 @@
       <c r="W28" s="3" t="n">
         <v>0.1000625</v>
       </c>
+      <c r="X28" s="3" t="n">
+        <v>0.1005625</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2686,6 +2770,9 @@
       <c r="W29" s="3" t="n">
         <v>0.10025</v>
       </c>
+      <c r="X29" s="3" t="n">
+        <v>0.1006666666666667</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2761,6 +2848,9 @@
       <c r="W30" s="3" t="n">
         <v>0.1006571428571429</v>
       </c>
+      <c r="X30" s="3" t="n">
+        <v>0.1012285714285714</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2836,6 +2926,9 @@
       <c r="W31" s="3" t="n">
         <v>0.1012</v>
       </c>
+      <c r="X31" s="3" t="n">
+        <v>0.1016166666666667</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2911,6 +3004,9 @@
       <c r="W32" s="3" t="n">
         <v>0.1018571428571429</v>
       </c>
+      <c r="X32" s="3" t="n">
+        <v>0.1025714285714286</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2986,6 +3082,9 @@
       <c r="W33" s="3" t="n">
         <v>0.1021666666666667</v>
       </c>
+      <c r="X33" s="3" t="n">
+        <v>0.10275</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3061,6 +3160,9 @@
       <c r="W34" s="3" t="n">
         <v>0.1027</v>
       </c>
+      <c r="X34" s="3" t="n">
+        <v>0.1028</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3136,6 +3238,9 @@
       <c r="W35" s="3" t="n">
         <v>0.1052</v>
       </c>
+      <c r="X35" s="3" t="n">
+        <v>0.1048</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3211,6 +3316,9 @@
       <c r="W36" s="3" t="n">
         <v>0.10675</v>
       </c>
+      <c r="X36" s="3" t="n">
+        <v>0.1066666666666667</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3286,6 +3394,9 @@
       <c r="W37" s="3" t="n">
         <v>0.1074125</v>
       </c>
+      <c r="X37" s="3" t="n">
+        <v>0.10785</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3361,6 +3472,9 @@
       <c r="W38" s="3" t="n">
         <v>0.1076777777777778</v>
       </c>
+      <c r="X38" s="3" t="n">
+        <v>0.1081777777777778</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3436,6 +3550,9 @@
       <c r="W39" s="3" t="n">
         <v>0.10888</v>
       </c>
+      <c r="X39" s="3" t="n">
+        <v>0.10868</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3511,6 +3628,9 @@
       <c r="W40" s="3" t="n">
         <v>0.1094625</v>
       </c>
+      <c r="X40" s="3" t="n">
+        <v>0.1100875</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3586,6 +3706,9 @@
       <c r="W41" s="3" t="n">
         <v>0.1093833333333333</v>
       </c>
+      <c r="X41" s="3" t="n">
+        <v>0.1098833333333333</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3661,6 +3784,9 @@
       <c r="W42" s="3" t="n">
         <v>0.1098125</v>
       </c>
+      <c r="X42" s="3" t="n">
+        <v>0.1104375</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3736,6 +3862,9 @@
       <c r="W43" s="3" t="n">
         <v>0.11042</v>
       </c>
+      <c r="X43" s="3" t="n">
+        <v>0.11052</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3811,6 +3940,9 @@
       <c r="W44" s="3" t="n">
         <v>0.1112555555555556</v>
       </c>
+      <c r="X44" s="3" t="n">
+        <v>0.1119777777777778</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3886,6 +4018,9 @@
       <c r="W45" s="3" t="n">
         <v>0.1109</v>
       </c>
+      <c r="X45" s="3" t="n">
+        <v>0.1114</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3961,6 +4096,9 @@
       <c r="W46" s="3" t="n">
         <v>0.11174</v>
       </c>
+      <c r="X46" s="3" t="n">
+        <v>0.11204</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4036,6 +4174,9 @@
       <c r="W47" s="3" t="n">
         <v>0.1121</v>
       </c>
+      <c r="X47" s="3" t="n">
+        <v>0.112775</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4111,6 +4252,9 @@
       <c r="W48" s="3" t="n">
         <v>0.1122857142857143</v>
       </c>
+      <c r="X48" s="3" t="n">
+        <v>0.1125714285714286</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4186,6 +4330,9 @@
       <c r="W49" s="3" t="n">
         <v>0.1124166666666667</v>
       </c>
+      <c r="X49" s="3" t="n">
+        <v>0.1126666666666667</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4261,6 +4408,9 @@
       <c r="W50" s="3" t="n">
         <v>0.1127857142857143</v>
       </c>
+      <c r="X50" s="3" t="n">
+        <v>0.113</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4336,6 +4486,9 @@
       <c r="W51" s="3" t="n">
         <v>0.114</v>
       </c>
+      <c r="X51" s="3" t="n">
+        <v>0.114125</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4411,6 +4564,9 @@
       <c r="W52" s="3" t="n">
         <v>0.1145</v>
       </c>
+      <c r="X52" s="3" t="n">
+        <v>0.114625</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4486,6 +4642,9 @@
       <c r="W53" s="3" t="n">
         <v>0.115</v>
       </c>
+      <c r="X53" s="3" t="n">
+        <v>0.115125</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4561,6 +4720,9 @@
       <c r="W54" s="3" t="n">
         <v>0.115875</v>
       </c>
+      <c r="X54" s="3" t="n">
+        <v>0.116</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4635,6 +4797,9 @@
       </c>
       <c r="W55" s="3" t="n">
         <v>0.1166666666666667</v>
+      </c>
+      <c r="X55" s="3" t="n">
+        <v>0.1165</v>
       </c>
     </row>
     <row r="56">
@@ -4675,6 +4840,9 @@
       <c r="W56" s="3" t="n">
         <v>0.1009833333333334</v>
       </c>
+      <c r="X56" s="3" t="n">
+        <v>0.1017</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4687,7 +4855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W40"/>
+  <dimension ref="A1:X40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4713,6 +4881,7 @@
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4831,6 +5000,11 @@
           <t>14-May-26</t>
         </is>
       </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>18-May-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4906,6 +5080,9 @@
       <c r="W2" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X2" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4981,6 +5158,9 @@
       <c r="W3" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="X3" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -5056,6 +5236,9 @@
       <c r="W4" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X4" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -5131,6 +5314,9 @@
       <c r="W5" s="3" t="n">
         <v>0.13005</v>
       </c>
+      <c r="X5" s="3" t="n">
+        <v>0.13005</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -5206,6 +5392,9 @@
       <c r="W6" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X6" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -5281,6 +5470,9 @@
       <c r="W7" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X7" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -5356,6 +5548,9 @@
       <c r="W8" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X8" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -5431,6 +5626,9 @@
       <c r="W9" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X9" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -5506,6 +5704,9 @@
       <c r="W10" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X10" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -5581,6 +5782,9 @@
       <c r="W11" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X11" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5656,6 +5860,9 @@
       <c r="W12" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X12" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5731,6 +5938,9 @@
       <c r="W13" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X13" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5806,6 +6016,9 @@
       <c r="W14" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X14" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5881,6 +6094,9 @@
       <c r="W15" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X15" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5956,6 +6172,9 @@
       <c r="W16" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X16" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6031,6 +6250,9 @@
       <c r="W17" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X17" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6106,6 +6328,9 @@
       <c r="W18" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X18" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6181,6 +6406,9 @@
       <c r="W19" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X19" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6256,6 +6484,9 @@
       <c r="W20" s="3" t="n">
         <v>0.08666666666666667</v>
       </c>
+      <c r="X20" s="3" t="n">
+        <v>0.08666666666666667</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6331,6 +6562,9 @@
       <c r="W21" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X21" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6406,6 +6640,9 @@
       <c r="W22" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X22" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6481,6 +6718,9 @@
       <c r="W23" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X23" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6556,6 +6796,9 @@
       <c r="W24" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X24" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6631,6 +6874,9 @@
       <c r="W25" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X25" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6706,6 +6952,9 @@
       <c r="W26" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X26" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6781,6 +7030,9 @@
       <c r="W27" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X27" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -6856,6 +7108,9 @@
       <c r="W28" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X28" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -6931,6 +7186,9 @@
       <c r="W29" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X29" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7006,6 +7264,9 @@
       <c r="W30" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X30" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7081,6 +7342,9 @@
       <c r="W31" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X31" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -7156,6 +7420,9 @@
       <c r="W32" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X32" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -7231,6 +7498,9 @@
       <c r="W33" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X33" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -7306,6 +7576,9 @@
       <c r="W34" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X34" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -7381,6 +7654,9 @@
       <c r="W35" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X35" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -7456,6 +7732,9 @@
       <c r="W36" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X36" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -7531,6 +7810,9 @@
       <c r="W37" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X37" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -7606,6 +7888,9 @@
       <c r="W38" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X38" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7681,6 +7966,9 @@
       <c r="W39" s="3" t="n">
         <v>0.13</v>
       </c>
+      <c r="X39" s="3" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7754,6 +8042,9 @@
         <v>0.13</v>
       </c>
       <c r="W40" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="X40" s="3" t="n">
         <v>0.13</v>
       </c>
     </row>

</xml_diff>